<commit_message>
fix: align v0.9.3 score comparison columns
</commit_message>
<xml_diff>
--- a/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.9.3-rescored.xlsx
+++ b/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.9.3-rescored.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="Re662f0a8e33546ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="R73f0e14cba0d434e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -419,7 +419,7 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="79">
+  <x:cellXfs count="78">
     <x:xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -653,9 +653,6 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
-    </x:xf>
-    <x:xf numFmtId="59" fontId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
-      <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -918,10 +915,6 @@
       <x:c r="N1"/>
       <x:c r="O1"/>
       <x:c r="P1"/>
-      <x:c r="Q1"/>
-      <x:c r="R1"/>
-      <x:c r="S1"/>
-      <x:c r="T1"/>
     </x:row>
     <x:row r="2" ht="22.350000381469727" customHeight="1">
       <x:c r="A2" s="5" t="str">
@@ -956,18 +949,6 @@
       </x:c>
       <x:c r="O2" s="62"/>
       <x:c r="P2" s="62"/>
-      <x:c r="Q2" t="str">
-        <x:v>gpt-5-6-sol</x:v>
-      </x:c>
-      <x:c r="R2" t="str">
-        <x:v>gpt-5-6-sol</x:v>
-      </x:c>
-      <x:c r="S2" t="str">
-        <x:v>qwen3-8-flash</x:v>
-      </x:c>
-      <x:c r="T2" t="str">
-        <x:v>qwen3-8-flash</x:v>
-      </x:c>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="6"/>
@@ -994,18 +975,6 @@
       </x:c>
       <x:c r="O3" s="62"/>
       <x:c r="P3" s="62"/>
-      <x:c r="Q3" t="str">
-        <x:v>skill-on</x:v>
-      </x:c>
-      <x:c r="R3" t="str">
-        <x:v>skill-off</x:v>
-      </x:c>
-      <x:c r="S3" t="str">
-        <x:v>skill-on</x:v>
-      </x:c>
-      <x:c r="T3" t="str">
-        <x:v>skill-off</x:v>
-      </x:c>
     </x:row>
     <x:row r="4" ht="22.5" customHeight="1">
       <x:c r="A4" s="7"/>
@@ -1016,48 +985,36 @@
         <x:v>作答结果</x:v>
       </x:c>
       <x:c r="F4" s="8" t="str">
-        <x:v>v0.9.1 得分</x:v>
+        <x:v>v0.9.2 得分</x:v>
       </x:c>
       <x:c r="G4" s="8" t="str">
-        <x:v>v0.9.2 得分</x:v>
+        <x:v>v0.9.3 得分</x:v>
       </x:c>
       <x:c r="H4" s="8" t="str">
         <x:v>作答结果</x:v>
       </x:c>
       <x:c r="I4" s="8" t="str">
-        <x:v>v0.9.1 得分</x:v>
+        <x:v>v0.9.2 得分</x:v>
       </x:c>
       <x:c r="J4" s="8" t="str">
-        <x:v>v0.9.2 得分</x:v>
+        <x:v>v0.9.3 得分</x:v>
       </x:c>
       <x:c r="K4" s="8" t="str">
         <x:v>作答结果</x:v>
       </x:c>
       <x:c r="L4" s="8" t="str">
-        <x:v>v0.9.1 得分</x:v>
+        <x:v>v0.9.2 得分</x:v>
       </x:c>
       <x:c r="M4" s="63" t="str">
-        <x:v>v0.9.2 得分</x:v>
+        <x:v>v0.9.3 得分</x:v>
       </x:c>
       <x:c r="N4" s="63" t="str">
         <x:v>作答结果</x:v>
       </x:c>
       <x:c r="O4" s="63" t="str">
-        <x:v>v0.9.1 得分</x:v>
+        <x:v>v0.9.2 得分</x:v>
       </x:c>
       <x:c r="P4" s="63" t="str">
-        <x:v>v0.9.2 得分</x:v>
-      </x:c>
-      <x:c r="Q4" t="str">
-        <x:v>v0.9.3 得分</x:v>
-      </x:c>
-      <x:c r="R4" t="str">
-        <x:v>v0.9.3 得分</x:v>
-      </x:c>
-      <x:c r="S4" t="str">
-        <x:v>v0.9.3 得分</x:v>
-      </x:c>
-      <x:c r="T4" t="str">
         <x:v>v0.9.3 得分</x:v>
       </x:c>
     </x:row>
@@ -1081,7 +1038,7 @@
         <x:v>0.982187</x:v>
       </x:c>
       <x:c r="G5" s="23" t="n">
-        <x:v>0.982187</x:v>
+        <x:v>0.977733540125</x:v>
       </x:c>
       <x:c r="H5" s="11" t="str">
         <x:v>{"answer":90.35,"unit":"kJ/mol"}</x:v>
@@ -1099,7 +1056,7 @@
         <x:v>0.982197</x:v>
       </x:c>
       <x:c r="M5" s="65" t="n">
-        <x:v>0.982197</x:v>
+        <x:v>0.977746040125</x:v>
       </x:c>
       <x:c r="N5" s="67" t="str">
         <x:v>{"answer":2.81,"unit":"kJ/mol"}</x:v>
@@ -1108,18 +1065,6 @@
         <x:v>0.744803</x:v>
       </x:c>
       <x:c r="P5" s="65" t="n">
-        <x:v>0.744803</x:v>
-      </x:c>
-      <x:c r="Q5" s="78" t="n">
-        <x:v>0.977733540125</x:v>
-      </x:c>
-      <x:c r="R5" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S5" s="78" t="n">
-        <x:v>0.977746040125</x:v>
-      </x:c>
-      <x:c r="T5" s="78" t="n">
         <x:v>0.681003959875</x:v>
       </x:c>
     </x:row>
@@ -1140,48 +1085,36 @@
         <x:v>{"answers":[{"property":"potential_energy_difference","value":7.299201259709321,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
       <x:c r="F6" s="24" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.666667</x:v>
       </x:c>
       <x:c r="G6" s="24" t="n">
-        <x:v>0.666667</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="H6" s="14" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":5.50986,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
       <x:c r="I6" s="24" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.666667</x:v>
       </x:c>
       <x:c r="J6" s="24" t="n">
-        <x:v>0.666667</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="K6" s="14" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":5.51,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
       <x:c r="L6" s="24" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.666667</x:v>
       </x:c>
       <x:c r="M6" s="69" t="n">
-        <x:v>0.666667</x:v>
+        <x:v>0.6666666666666666</x:v>
       </x:c>
       <x:c r="N6" s="71" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":7.17,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
       <x:c r="O6" s="69" t="n">
-        <x:v>0.5</x:v>
+        <x:v>0.666667</x:v>
       </x:c>
       <x:c r="P6" s="69" t="n">
-        <x:v>0.666667</x:v>
-      </x:c>
-      <x:c r="Q6" s="78" t="n">
-        <x:v>0.6666666666666666</x:v>
-      </x:c>
-      <x:c r="R6" s="78" t="n">
-        <x:v>0.6666666666666666</x:v>
-      </x:c>
-      <x:c r="S6" s="78" t="n">
-        <x:v>0.6666666666666666</x:v>
-      </x:c>
-      <x:c r="T6" s="78" t="n">
         <x:v>0.6666666666666666</x:v>
       </x:c>
     </x:row>
@@ -1232,18 +1165,6 @@
         <x:v>0.333333</x:v>
       </x:c>
       <x:c r="P7" s="69" t="n">
-        <x:v>0.333333</x:v>
-      </x:c>
-      <x:c r="Q7" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R7" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S7" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T7" s="78" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1264,19 +1185,19 @@
         <x:v>{"answers":[{"property":"frequency_1","value":435.81,"unit":"cm^-1"},{"property":"frequency_2","value":1585.74,"unit":"cm^-1"},{"property":"frequency_3","value":1592.57,"unit":"cm^-1"}]}</x:v>
       </x:c>
       <x:c r="F8" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>0.0009</x:v>
       </x:c>
       <x:c r="G8" s="24" t="n">
-        <x:v>0.0009</x:v>
+        <x:v>0.000900000000000345</x:v>
       </x:c>
       <x:c r="H8" s="14" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1585.71,"unit":"cm^-1"},{"property":"frequency_2","value":436.11,"unit":"cm^-1"},{"property":"frequency_3","value":1592.37,"unit":"cm^-1"}]}</x:v>
       </x:c>
       <x:c r="I8" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>0.00075</x:v>
       </x:c>
       <x:c r="J8" s="24" t="n">
-        <x:v>0.00075</x:v>
+        <x:v>0.0007500000000004725</x:v>
       </x:c>
       <x:c r="K8" s="14" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1584.79,"unit":"cm^-1"},{"property":"frequency_2","value":433.87,"unit":"cm^-1"},{"property":"frequency_3","value":1592.2,"unit":"cm^-1"}]}</x:v>
@@ -1291,21 +1212,9 @@
         <x:v>{"answers":[{"property":"frequency_1","value":1624.6,"unit":"cm^-1"},{"property":"frequency_2","value":1246.4,"unit":"cm^-1"},{"property":"frequency_3","value":843.1,"unit":"cm^-1"}]}</x:v>
       </x:c>
       <x:c r="O8" s="69" t="n">
-        <x:v>0.3904</x:v>
+        <x:v>0.5037</x:v>
       </x:c>
       <x:c r="P8" s="69" t="n">
-        <x:v>0.5037</x:v>
-      </x:c>
-      <x:c r="Q8" s="78" t="n">
-        <x:v>0.000900000000000345</x:v>
-      </x:c>
-      <x:c r="R8" s="78" t="n">
-        <x:v>0.0007500000000004725</x:v>
-      </x:c>
-      <x:c r="S8" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T8" s="78" t="n">
         <x:v>0.5036999999999989</x:v>
       </x:c>
     </x:row>
@@ -1329,7 +1238,7 @@
         <x:v>0.4864</x:v>
       </x:c>
       <x:c r="G9" s="24" t="n">
-        <x:v>0.4864</x:v>
+        <x:v>0.2902548228400852</x:v>
       </x:c>
       <x:c r="H9" s="14" t="str">
         <x:v>{"answer":1.56,"unit":"g/cm^3"}</x:v>
@@ -1338,7 +1247,7 @@
         <x:v>0.4364</x:v>
       </x:c>
       <x:c r="J9" s="24" t="n">
-        <x:v>0.4364</x:v>
+        <x:v>0.2211596926648599</x:v>
       </x:c>
       <x:c r="K9" s="14" t="str">
         <x:v>{"answer":1.47,"unit":"g/cm^3"}</x:v>
@@ -1347,7 +1256,7 @@
         <x:v>0.8864</x:v>
       </x:c>
       <x:c r="M9" s="69" t="n">
-        <x:v>0.8864</x:v>
+        <x:v>0.8430158642418877</x:v>
       </x:c>
       <x:c r="N9" s="71" t="str">
         <x:v>{"answer":1.28,"unit":"g/cm^3"}</x:v>
@@ -1356,18 +1265,6 @@
         <x:v>0.1636</x:v>
       </x:c>
       <x:c r="P9" s="69" t="n">
-        <x:v>0.1636</x:v>
-      </x:c>
-      <x:c r="Q9" s="78" t="n">
-        <x:v>0.2902548228400852</x:v>
-      </x:c>
-      <x:c r="R9" s="78" t="n">
-        <x:v>0.2211596926648599</x:v>
-      </x:c>
-      <x:c r="S9" s="78" t="n">
-        <x:v>0.8430158642418877</x:v>
-      </x:c>
-      <x:c r="T9" s="78" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1420,18 +1317,6 @@
       <x:c r="P10" s="69" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="Q10" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R10" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="S10" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T10" s="78" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
     </x:row>
     <x:row r="11" ht="68.05000305175781" customHeight="1">
       <x:c r="A11" s="12" t="str">
@@ -1459,7 +1344,7 @@
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormC"},{"property":"crossover_temperature","value":943,"unit":"K"}]}</x:v>
       </x:c>
       <x:c r="I11" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="J11" s="24" t="n">
         <x:v>0.5</x:v>
@@ -1468,30 +1353,18 @@
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":428.5,"unit":"K"}]}</x:v>
       </x:c>
       <x:c r="L11" s="24" t="n">
-        <x:v>0</x:v>
+        <x:v>0.286625</x:v>
       </x:c>
       <x:c r="M11" s="69" t="n">
-        <x:v>0.286625</x:v>
+        <x:v>0.07324999999999987</x:v>
       </x:c>
       <x:c r="N11" s="71" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":300,"unit":"K"}]}</x:v>
       </x:c>
       <x:c r="O11" s="69" t="n">
-        <x:v>0</x:v>
+        <x:v>0.392125</x:v>
       </x:c>
       <x:c r="P11" s="69" t="n">
-        <x:v>0.392125</x:v>
-      </x:c>
-      <x:c r="Q11" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R11" s="78" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="S11" s="78" t="n">
-        <x:v>0.07324999999999987</x:v>
-      </x:c>
-      <x:c r="T11" s="78" t="n">
         <x:v>0.2842500000000001</x:v>
       </x:c>
     </x:row>
@@ -1512,48 +1385,36 @@
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.4733,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.3678,"unit":"kcal/mol"}]}</x:v>
       </x:c>
       <x:c r="F12" s="24" t="n">
-        <x:v>0.928335</x:v>
+        <x:v>0.933723</x:v>
       </x:c>
       <x:c r="G12" s="24" t="n">
-        <x:v>0.933723</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H12" s="14" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.47,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.38,"unit":"kcal/mol"}]}</x:v>
       </x:c>
       <x:c r="I12" s="24" t="n">
-        <x:v>0.9285</x:v>
+        <x:v>0.9335</x:v>
       </x:c>
       <x:c r="J12" s="24" t="n">
-        <x:v>0.9335</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K12" s="14" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.45,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.37,"unit":"kcal/mol"}]}</x:v>
       </x:c>
       <x:c r="L12" s="24" t="n">
-        <x:v>0.9295</x:v>
+        <x:v>0.93425</x:v>
       </x:c>
       <x:c r="M12" s="69" t="n">
-        <x:v>0.93425</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N12" s="71" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.49,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.38,"unit":"kcal/mol"}]}</x:v>
       </x:c>
       <x:c r="O12" s="69" t="n">
-        <x:v>0.9275</x:v>
+        <x:v>0.933</x:v>
       </x:c>
       <x:c r="P12" s="69" t="n">
-        <x:v>0.933</x:v>
-      </x:c>
-      <x:c r="Q12" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R12" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S12" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T12" s="78" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1606,18 +1467,6 @@
       <x:c r="P13" s="69" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q13" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R13" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S13" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T13" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
     </x:row>
     <x:row r="14" ht="68.05000305175781" customHeight="1">
       <x:c r="A14" s="12" t="str">
@@ -1636,48 +1485,36 @@
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
       <x:c r="F14" s="24" t="n">
-        <x:v>0.643333</x:v>
+        <x:v>0.776667</x:v>
       </x:c>
       <x:c r="G14" s="24" t="n">
-        <x:v>0.776667</x:v>
+        <x:v>0.6650000000000003</x:v>
       </x:c>
       <x:c r="H14" s="14" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.001520301,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.594671850,"unit":"angstrom"}]}</x:v>
       </x:c>
       <x:c r="I14" s="24" t="n">
-        <x:v>0.634427</x:v>
+        <x:v>0.771414</x:v>
       </x:c>
       <x:c r="J14" s="24" t="n">
-        <x:v>0.771414</x:v>
+        <x:v>0.6571211275000007</x:v>
       </x:c>
       <x:c r="K14" s="14" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
       <x:c r="L14" s="24" t="n">
-        <x:v>0.643333</x:v>
+        <x:v>0.776667</x:v>
       </x:c>
       <x:c r="M14" s="69" t="n">
-        <x:v>0.776667</x:v>
+        <x:v>0.6650000000000003</x:v>
       </x:c>
       <x:c r="N14" s="71" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
       <x:c r="O14" s="69" t="n">
-        <x:v>0.643333</x:v>
+        <x:v>0.776667</x:v>
       </x:c>
       <x:c r="P14" s="69" t="n">
-        <x:v>0.776667</x:v>
-      </x:c>
-      <x:c r="Q14" s="78" t="n">
-        <x:v>0.6650000000000003</x:v>
-      </x:c>
-      <x:c r="R14" s="78" t="n">
-        <x:v>0.6571211275000007</x:v>
-      </x:c>
-      <x:c r="S14" s="78" t="n">
-        <x:v>0.6650000000000003</x:v>
-      </x:c>
-      <x:c r="T14" s="78" t="n">
         <x:v>0.6650000000000003</x:v>
       </x:c>
     </x:row>
@@ -1730,18 +1567,6 @@
       <x:c r="P15" s="69" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="Q15" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R15" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S15" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T15" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
     </x:row>
     <x:row r="16" ht="65.1500015258789" customHeight="1">
       <x:c r="A16" s="12" t="str">
@@ -1763,7 +1588,7 @@
         <x:v>0.9996</x:v>
       </x:c>
       <x:c r="G16" s="24" t="n">
-        <x:v>0.9996</x:v>
+        <x:v>0.9990000000000001</x:v>
       </x:c>
       <x:c r="H16" s="14" t="str">
         <x:v>{"answer":2.5183,"unit":"angstrom"}</x:v>
@@ -1772,7 +1597,7 @@
         <x:v>0.9946</x:v>
       </x:c>
       <x:c r="J16" s="24" t="n">
-        <x:v>0.9946</x:v>
+        <x:v>0.9865000000000004</x:v>
       </x:c>
       <x:c r="K16" s="14" t="str">
         <x:v>{"answer":2.52,"unit":"angstrom"}</x:v>
@@ -1781,7 +1606,7 @@
         <x:v>0.998</x:v>
       </x:c>
       <x:c r="M16" s="69" t="n">
-        <x:v>0.998</x:v>
+        <x:v>0.9950000000000006</x:v>
       </x:c>
       <x:c r="N16" s="71" t="str">
         <x:v>{"answer":2.7043,"unit":"angstrom"}</x:v>
@@ -1790,18 +1615,6 @@
         <x:v>0.6334</x:v>
       </x:c>
       <x:c r="P16" s="69" t="n">
-        <x:v>0.6334</x:v>
-      </x:c>
-      <x:c r="Q16" s="78" t="n">
-        <x:v>0.9990000000000001</x:v>
-      </x:c>
-      <x:c r="R16" s="78" t="n">
-        <x:v>0.9865000000000004</x:v>
-      </x:c>
-      <x:c r="S16" s="78" t="n">
-        <x:v>0.9950000000000006</x:v>
-      </x:c>
-      <x:c r="T16" s="78" t="n">
         <x:v>0.08349999999999991</x:v>
       </x:c>
     </x:row>
@@ -1834,7 +1647,7 @@
         <x:v>0.588</x:v>
       </x:c>
       <x:c r="J17" s="24" t="n">
-        <x:v>0.588</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K17" s="14" t="str">
         <x:v>{"answer":-15.5969,"unit":"kcal/mol"}</x:v>
@@ -1843,7 +1656,7 @@
         <x:v>0.69738</x:v>
       </x:c>
       <x:c r="M17" s="69" t="n">
-        <x:v>0.69738</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N17" s="71" t="str">
         <x:v>{"answer":-16.5,"unit":"kcal/mol"}</x:v>
@@ -1852,18 +1665,6 @@
         <x:v>0.878</x:v>
       </x:c>
       <x:c r="P17" s="69" t="n">
-        <x:v>0.878</x:v>
-      </x:c>
-      <x:c r="Q17" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R17" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S17" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T17" s="78" t="n">
         <x:v>0.39000000000000057</x:v>
       </x:c>
     </x:row>
@@ -1887,7 +1688,7 @@
         <x:v>0.65</x:v>
       </x:c>
       <x:c r="G18" s="24" t="n">
-        <x:v>0.65</x:v>
+        <x:v>0.6499999999999999</x:v>
       </x:c>
       <x:c r="H18" s="14" t="str">
         <x:v>{"answer":6.33,"unit":"pKa"}</x:v>
@@ -1914,18 +1715,6 @@
         <x:v>0.45</x:v>
       </x:c>
       <x:c r="P18" s="69" t="n">
-        <x:v>0.45</x:v>
-      </x:c>
-      <x:c r="Q18" s="78" t="n">
-        <x:v>0.6499999999999999</x:v>
-      </x:c>
-      <x:c r="R18" s="78" t="n">
-        <x:v>0.685</x:v>
-      </x:c>
-      <x:c r="S18" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T18" s="78" t="n">
         <x:v>0.4500000000000002</x:v>
       </x:c>
     </x:row>
@@ -1949,7 +1738,7 @@
         <x:v>0.820046</x:v>
       </x:c>
       <x:c r="G19" s="24" t="n">
-        <x:v>0.820046</x:v>
+        <x:v>0.8200456786861929</x:v>
       </x:c>
       <x:c r="H19" s="14" t="str">
         <x:v>{"answer":0.0035,"unit":"eV"}</x:v>
@@ -1958,7 +1747,7 @@
         <x:v>0.678372</x:v>
       </x:c>
       <x:c r="J19" s="24" t="n">
-        <x:v>0.678372</x:v>
+        <x:v>0.6783719844342051</x:v>
       </x:c>
       <x:c r="K19" s="14" t="str">
         <x:v>{"answer":0.0,"unit":"eV"}</x:v>
@@ -1976,18 +1765,6 @@
         <x:v>0.865696</x:v>
       </x:c>
       <x:c r="P19" s="69" t="n">
-        <x:v>0.865696</x:v>
-      </x:c>
-      <x:c r="Q19" s="78" t="n">
-        <x:v>0.8200456786861929</x:v>
-      </x:c>
-      <x:c r="R19" s="78" t="n">
-        <x:v>0.6783719844342051</x:v>
-      </x:c>
-      <x:c r="S19" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T19" s="78" t="n">
         <x:v>0.8656960599160706</x:v>
       </x:c>
     </x:row>
@@ -2011,7 +1788,7 @@
         <x:v>0.996335</x:v>
       </x:c>
       <x:c r="G20" s="24" t="n">
-        <x:v>0.996335</x:v>
+        <x:v>0.9945023078492685</x:v>
       </x:c>
       <x:c r="H20" s="14" t="str">
         <x:v>{"answer":1.45e8,"unit":"s^-1"}</x:v>
@@ -2020,7 +1797,7 @@
         <x:v>0.968939</x:v>
       </x:c>
       <x:c r="J20" s="24" t="n">
-        <x:v>0.968939</x:v>
+        <x:v>0.9534089297555939</x:v>
       </x:c>
       <x:c r="K20" s="14" t="str">
         <x:v>{"answer":1e6,"unit":"s^-1"}</x:v>
@@ -2029,7 +1806,7 @@
         <x:v>0.310605</x:v>
       </x:c>
       <x:c r="M20" s="69" t="n">
-        <x:v>0.310605</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="N20" s="71" t="str">
         <x:v>{"answer":100000,"unit":"s^-1"}</x:v>
@@ -2038,18 +1815,6 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="P20" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q20" s="78" t="n">
-        <x:v>0.9945023078492685</x:v>
-      </x:c>
-      <x:c r="R20" s="78" t="n">
-        <x:v>0.9534089297555939</x:v>
-      </x:c>
-      <x:c r="S20" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="T20" s="78" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2073,7 +1838,7 @@
         <x:v>0.986111</x:v>
       </x:c>
       <x:c r="G21" s="24" t="n">
-        <x:v>0.986111</x:v>
+        <x:v>0.9861105136520333</x:v>
       </x:c>
       <x:c r="H21" s="14" t="str">
         <x:v>{"answer":100.0,"unit":"s^-1"}</x:v>
@@ -2082,7 +1847,7 @@
         <x:v>0.997075</x:v>
       </x:c>
       <x:c r="J21" s="24" t="n">
-        <x:v>0.997075</x:v>
+        <x:v>0.9956130378462474</x:v>
       </x:c>
       <x:c r="K21" s="14" t="str">
         <x:v>{"answer":100,"unit":"s^-1"}</x:v>
@@ -2091,7 +1856,7 @@
         <x:v>0.997075</x:v>
       </x:c>
       <x:c r="M21" s="69" t="n">
-        <x:v>0.997075</x:v>
+        <x:v>0.9956130378462474</x:v>
       </x:c>
       <x:c r="N21" s="71" t="str">
         <x:v>{"answer":16.9,"unit":"s^-1"}</x:v>
@@ -2100,18 +1865,6 @@
         <x:v>0.61833</x:v>
       </x:c>
       <x:c r="P21" s="69" t="n">
-        <x:v>0.61833</x:v>
-      </x:c>
-      <x:c r="Q21" s="78" t="n">
-        <x:v>0.9861105136520333</x:v>
-      </x:c>
-      <x:c r="R21" s="78" t="n">
-        <x:v>0.9956130378462474</x:v>
-      </x:c>
-      <x:c r="S21" s="78" t="n">
-        <x:v>0.9956130378462474</x:v>
-      </x:c>
-      <x:c r="T21" s="78" t="n">
         <x:v>0.6183303144605893</x:v>
       </x:c>
     </x:row>
@@ -2164,18 +1917,6 @@
       <x:c r="P22" s="69" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="Q22" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="R22" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S22" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="T22" s="78" t="n">
-        <x:v>1</x:v>
-      </x:c>
     </x:row>
     <x:row r="23" ht="79.4000015258789" customHeight="1">
       <x:c r="A23" s="12" t="str">
@@ -2197,7 +1938,7 @@
         <x:v>0.97442</x:v>
       </x:c>
       <x:c r="G23" s="24" t="n">
-        <x:v>0.97442</x:v>
+        <x:v>0.9616293085047376</x:v>
       </x:c>
       <x:c r="H23" s="14" t="str">
         <x:v>{"answer":1.6e8,"unit":"s^-1"}</x:v>
@@ -2206,7 +1947,7 @@
         <x:v>0.250267</x:v>
       </x:c>
       <x:c r="J23" s="24" t="n">
-        <x:v>0.250267</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="K23" s="14" t="str">
         <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
@@ -2215,7 +1956,7 @@
         <x:v>0.848894</x:v>
       </x:c>
       <x:c r="M23" s="69" t="n">
-        <x:v>0.848894</x:v>
+        <x:v>0.7733408299764815</x:v>
       </x:c>
       <x:c r="N23" s="71" t="str">
         <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
@@ -2224,18 +1965,6 @@
         <x:v>0.848894</x:v>
       </x:c>
       <x:c r="P23" s="69" t="n">
-        <x:v>0.848894</x:v>
-      </x:c>
-      <x:c r="Q23" s="78" t="n">
-        <x:v>0.9616293085047376</x:v>
-      </x:c>
-      <x:c r="R23" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S23" s="78" t="n">
-        <x:v>0.7733408299764815</x:v>
-      </x:c>
-      <x:c r="T23" s="78" t="n">
         <x:v>0.7733408299764815</x:v>
       </x:c>
     </x:row>
@@ -2277,23 +2006,13 @@
         <x:v>0.860688</x:v>
       </x:c>
       <x:c r="M24" s="74" t="n">
-        <x:v>0.860688</x:v>
+        <x:v>0.7910316814558547</x:v>
       </x:c>
       <x:c r="N24" s="75"/>
-      <x:c r="O24" s="74"/>
+      <x:c r="O24" s="74" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="P24" s="74" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="Q24" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="R24" s="78" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="S24" s="78" t="n">
-        <x:v>0.7910316814558547</x:v>
-      </x:c>
-      <x:c r="T24" s="78" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2308,48 +2027,36 @@
         <x:v>平均分</x:v>
       </x:c>
       <x:c r="F25" s="26" t="n">
-        <x:v>0.648338</x:v>
+        <x:v>0.663653</x:v>
       </x:c>
       <x:c r="G25" s="26" t="n">
-        <x:v>0.663653</x:v>
+        <x:v>0.6005921419161993</x:v>
       </x:c>
       <x:c r="H25" s="22" t="str">
         <x:v>平均分</x:v>
       </x:c>
       <x:c r="I25" s="26" t="n">
-        <x:v>0.483079</x:v>
+        <x:v>0.523549</x:v>
       </x:c>
       <x:c r="J25" s="26" t="n">
-        <x:v>0.523549</x:v>
+        <x:v>0.41722957194337873</x:v>
       </x:c>
       <x:c r="K25" s="21" t="str">
         <x:v>平均分</x:v>
       </x:c>
       <x:c r="L25" s="26" t="n">
-        <x:v>0.632704</x:v>
+        <x:v>0.662272</x:v>
       </x:c>
       <x:c r="M25" s="76" t="n">
-        <x:v>0.662272</x:v>
+        <x:v>0.5390332060156069</x:v>
       </x:c>
       <x:c r="N25" s="77" t="str">
         <x:v>平均分</x:v>
       </x:c>
       <x:c r="O25" s="76" t="n">
-        <x:v>0.474864</x:v>
+        <x:v>0.515411</x:v>
       </x:c>
       <x:c r="P25" s="76" t="n">
-        <x:v>0.515411</x:v>
-      </x:c>
-      <x:c r="Q25" s="78" t="n">
-        <x:v>0.6005921419161993</x:v>
-      </x:c>
-      <x:c r="R25" s="78" t="n">
-        <x:v>0.41722957194337873</x:v>
-      </x:c>
-      <x:c r="S25" s="78" t="n">
-        <x:v>0.5390332060156069</x:v>
-      </x:c>
-      <x:c r="T25" s="78" t="n">
         <x:v>0.37407439154474037</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
fix: remove question notes from score workbooks
</commit_message>
<xml_diff>
--- a/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.9.3-rescored.xlsx
+++ b/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.9.3-rescored.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="R73f0e14cba0d434e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="R785ec70e719f4c04"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -419,7 +419,7 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellStyleXfs>
-  <x:cellXfs count="78">
+  <x:cellXfs count="105">
     <x:xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -653,6 +653,87 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="8" fillId="11" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf fontId="4" fillId="3" borderId="4" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="4" fillId="4" borderId="6" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="4" fillId="4" borderId="9" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="4" fillId="4" borderId="11" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="5" fillId="5" borderId="14" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf fontId="0" fillId="2" borderId="7" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="0" fillId="2" borderId="10" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="0" fillId="2" borderId="12" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="0" fillId="2" borderId="8" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="0" fillId="2" borderId="4" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="0" fillId="2" borderId="13" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="4" fillId="3" borderId="5" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf fontId="5" fillId="5" borderId="14" xfId="0" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="59" fontId="5" fillId="5" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="7" fillId="7" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -877,1186 +958,1119 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultColWidth="16.33329963684082" defaultRowHeight="19.850000381469727"/>
   <x:cols>
-    <x:col min="1" max="1" width="23.171899795532227" style="1" customWidth="1"/>
-    <x:col min="2" max="2" width="29.171899795532227" style="1" customWidth="1"/>
-    <x:col min="3" max="3" width="26.171899795532227" style="1" customWidth="1"/>
-    <x:col min="4" max="4" width="29.851600646972656" style="1" customWidth="1"/>
-    <x:col min="5" max="5" width="19.351600646972656" style="1" customWidth="1"/>
-    <x:col min="6" max="6" width="12.35159969329834" style="1" customWidth="1"/>
-    <x:col min="7" max="7" width="18" style="1" customWidth="1"/>
-    <x:col min="8" max="8" width="13.5" style="1" customWidth="1"/>
-    <x:col min="9" max="9" width="17" style="1" customWidth="1"/>
-    <x:col min="10" max="10" width="12" style="1" customWidth="1"/>
-    <x:col min="11" max="11" width="17.5" style="1" customWidth="1"/>
-    <x:col min="12" max="12" width="16.351600646972656" style="1" customWidth="1"/>
+    <x:col min="1" max="1" width="23.171899795532227" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="26.171899795532227" style="1" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="29.851600646972656" style="1" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="19.351600646972656" style="1" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="12.35159969329834" style="1" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" style="1" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="13.5" style="1" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="17" style="1" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="12" style="1" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="17.5" style="1" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16.351600646972656" style="1" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="16.351600646972656" style="1" hidden="0" customWidth="1"/>
     <x:col min="13" max="16384" width="16.351600646972656" style="1" customWidth="1"/>
-    <x:col min="13" max="13" width="16.351600646972656" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="17.5" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="17.5" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="16.351600646972656" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="16.351600646972656" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="16.351600646972656" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="31" customHeight="1">
-      <x:c r="A1" s="2" t="str">
+      <x:c r="A1" s="79" t="str">
         <x:v>表格 1</x:v>
       </x:c>
-      <x:c r="B1" s="3"/>
-      <x:c r="C1" s="3"/>
-      <x:c r="D1" s="3"/>
-      <x:c r="E1" s="3"/>
-      <x:c r="F1" s="3"/>
-      <x:c r="G1" s="3"/>
-      <x:c r="H1" s="3"/>
-      <x:c r="I1" s="3"/>
-      <x:c r="J1" s="3"/>
-      <x:c r="K1" s="3"/>
-      <x:c r="L1" s="4"/>
-      <x:c r="M1"/>
-      <x:c r="N1"/>
-      <x:c r="O1"/>
-      <x:c r="P1"/>
+      <x:c r="B1" s="87"/>
+      <x:c r="C1" s="87"/>
+      <x:c r="D1" s="87"/>
+      <x:c r="E1" s="87"/>
+      <x:c r="F1" s="87"/>
+      <x:c r="G1" s="87"/>
+      <x:c r="H1" s="87"/>
+      <x:c r="I1" s="87"/>
+      <x:c r="J1" s="87"/>
+      <x:c r="K1" s="87"/>
+      <x:c r="L1" s="99"/>
+      <x:c r="M1" s="100"/>
+      <x:c r="N1" s="100"/>
+      <x:c r="O1" s="100"/>
     </x:row>
     <x:row r="2" ht="22.350000381469727" customHeight="1">
-      <x:c r="A2" s="5" t="str">
+      <x:c r="A2" s="80" t="str">
         <x:v>题目 ID + 一句话概括</x:v>
       </x:c>
-      <x:c r="B2" s="5" t="str">
-        <x:v>问题备注</x:v>
-      </x:c>
-      <x:c r="C2" s="5" t="str">
+      <x:c r="B2" s="80" t="str">
         <x:v>本题的标准答案</x:v>
       </x:c>
-      <x:c r="D2" s="5" t="str">
+      <x:c r="C2" s="80" t="str">
         <x:v>评分备注</x:v>
       </x:c>
-      <x:c r="E2" s="5" t="str">
+      <x:c r="D2" s="80" t="str">
         <x:v>gpt-5-6-sol</x:v>
       </x:c>
-      <x:c r="F2" s="6"/>
-      <x:c r="G2" s="5"/>
-      <x:c r="H2" s="6" t="str">
+      <x:c r="E2" s="81"/>
+      <x:c r="F2" s="80"/>
+      <x:c r="G2" s="81" t="str">
         <x:v>gpt-5-6-sol</x:v>
       </x:c>
-      <x:c r="I2" s="5"/>
-      <x:c r="J2" s="6"/>
-      <x:c r="K2" s="5" t="str">
+      <x:c r="H2" s="80"/>
+      <x:c r="I2" s="81"/>
+      <x:c r="J2" s="80" t="str">
         <x:v>qwen3-8-flash</x:v>
       </x:c>
-      <x:c r="L2" s="6"/>
-      <x:c r="M2" s="62"/>
-      <x:c r="N2" s="62" t="str">
+      <x:c r="K2" s="81"/>
+      <x:c r="L2" s="81"/>
+      <x:c r="M2" s="31" t="str">
         <x:v>qwen3-8-flash</x:v>
       </x:c>
-      <x:c r="O2" s="62"/>
-      <x:c r="P2" s="62"/>
+      <x:c r="N2" s="31"/>
+      <x:c r="O2" s="31"/>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
-      <x:c r="A3" s="6"/>
-      <x:c r="B3" s="6"/>
-      <x:c r="C3" s="6"/>
-      <x:c r="D3" s="6"/>
-      <x:c r="E3" s="5" t="str">
+      <x:c r="A3" s="81"/>
+      <x:c r="B3" s="81"/>
+      <x:c r="C3" s="81"/>
+      <x:c r="D3" s="80" t="str">
         <x:v>skill-on</x:v>
       </x:c>
-      <x:c r="F3" s="6"/>
-      <x:c r="G3" s="5"/>
-      <x:c r="H3" s="6" t="str">
+      <x:c r="E3" s="81"/>
+      <x:c r="F3" s="80"/>
+      <x:c r="G3" s="81" t="str">
         <x:v>skill-off</x:v>
       </x:c>
-      <x:c r="I3" s="5"/>
-      <x:c r="J3" s="6"/>
-      <x:c r="K3" s="5" t="str">
+      <x:c r="H3" s="80"/>
+      <x:c r="I3" s="81"/>
+      <x:c r="J3" s="80" t="str">
         <x:v>skill-on</x:v>
       </x:c>
-      <x:c r="L3" s="6"/>
-      <x:c r="M3" s="62"/>
-      <x:c r="N3" s="62" t="str">
+      <x:c r="K3" s="81"/>
+      <x:c r="L3" s="81"/>
+      <x:c r="M3" s="31" t="str">
         <x:v>skill-off</x:v>
       </x:c>
-      <x:c r="O3" s="62"/>
-      <x:c r="P3" s="62"/>
+      <x:c r="N3" s="31"/>
+      <x:c r="O3" s="31"/>
     </x:row>
     <x:row r="4" ht="22.5" customHeight="1">
-      <x:c r="A4" s="7"/>
-      <x:c r="B4" s="7"/>
-      <x:c r="C4" s="7"/>
-      <x:c r="D4" s="7"/>
-      <x:c r="E4" s="8" t="str">
+      <x:c r="A4" s="82"/>
+      <x:c r="B4" s="82"/>
+      <x:c r="C4" s="82"/>
+      <x:c r="D4" s="95" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="F4" s="8" t="str">
+      <x:c r="E4" s="95" t="str">
         <x:v>v0.9.2 得分</x:v>
       </x:c>
-      <x:c r="G4" s="8" t="str">
+      <x:c r="F4" s="95" t="str">
         <x:v>v0.9.3 得分</x:v>
       </x:c>
-      <x:c r="H4" s="8" t="str">
+      <x:c r="G4" s="95" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="I4" s="8" t="str">
+      <x:c r="H4" s="95" t="str">
         <x:v>v0.9.2 得分</x:v>
       </x:c>
-      <x:c r="J4" s="8" t="str">
+      <x:c r="I4" s="95" t="str">
         <x:v>v0.9.3 得分</x:v>
       </x:c>
-      <x:c r="K4" s="8" t="str">
+      <x:c r="J4" s="95" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="L4" s="8" t="str">
+      <x:c r="K4" s="95" t="str">
         <x:v>v0.9.2 得分</x:v>
       </x:c>
-      <x:c r="M4" s="63" t="str">
+      <x:c r="L4" s="82" t="str">
         <x:v>v0.9.3 得分</x:v>
       </x:c>
-      <x:c r="N4" s="63" t="str">
+      <x:c r="M4" s="33" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="O4" s="63" t="str">
+      <x:c r="N4" s="33" t="str">
         <x:v>v0.9.2 得分</x:v>
       </x:c>
-      <x:c r="P4" s="63" t="str">
+      <x:c r="O4" s="33" t="str">
         <x:v>v0.9.3 得分</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="79.6500015258789" customHeight="1">
-      <x:c r="A5" s="9" t="str">
+      <x:c r="A5" s="83" t="str">
         <x:v>property_calculation_advanced_001_free_energy；概括：计算两种分子晶体在 300 K 时的自由能绝对差。</x:v>
       </x:c>
-      <x:c r="B5" s="10" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C5" s="11" t="str">
+      <x:c r="B5" s="88" t="str">
         <x:v>{"answer":0.258031679,"unit":"kJ/mol"}</x:v>
       </x:c>
-      <x:c r="D5" s="11" t="str">
+      <x:c r="C5" s="92" t="str">
         <x:v>free_energy_difference：标准答案 0.258031679 kJ/mol；linear_goal_v2。满分：x=0.258031679。部分分：|x-0.258031679|&lt;10 按距离线性递减。0分：|x-0.258031679|≥10、单位不匹配或值无效。</x:v>
       </x:c>
-      <x:c r="E5" s="11" t="str">
+      <x:c r="D5" s="92" t="str">
         <x:v>{"answer":0.0799,"unit":"kJ/mol"}</x:v>
       </x:c>
+      <x:c r="E5" s="23" t="n">
+        <x:v>0.982187</x:v>
+      </x:c>
       <x:c r="F5" s="23" t="n">
-        <x:v>0.982187</x:v>
-      </x:c>
-      <x:c r="G5" s="23" t="n">
         <x:v>0.977733540125</x:v>
       </x:c>
-      <x:c r="H5" s="11" t="str">
+      <x:c r="G5" s="92" t="str">
         <x:v>{"answer":90.35,"unit":"kJ/mol"}</x:v>
       </x:c>
+      <x:c r="H5" s="23" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="I5" s="23" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J5" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K5" s="11" t="str">
+      <x:c r="J5" s="92" t="str">
         <x:v>{"answer":0.08,"unit":"kJ/mol"}</x:v>
       </x:c>
+      <x:c r="K5" s="23" t="n">
+        <x:v>0.982197</x:v>
+      </x:c>
       <x:c r="L5" s="23" t="n">
-        <x:v>0.982197</x:v>
-      </x:c>
-      <x:c r="M5" s="65" t="n">
         <x:v>0.977746040125</x:v>
       </x:c>
-      <x:c r="N5" s="67" t="str">
+      <x:c r="M5" s="101" t="str">
         <x:v>{"answer":2.81,"unit":"kJ/mol"}</x:v>
       </x:c>
-      <x:c r="O5" s="65" t="n">
+      <x:c r="N5" s="103" t="n">
         <x:v>0.744803</x:v>
       </x:c>
-      <x:c r="P5" s="65" t="n">
+      <x:c r="O5" s="103" t="n">
         <x:v>0.681003959875</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="93.6500015258789" customHeight="1">
-      <x:c r="A6" s="12" t="str">
+      <x:c r="A6" s="84" t="str">
         <x:v>property_calculation_advanced_002_crystal_phase；概括：计算 alpha/beta 晶相势能差并判断常压相和高压相。</x:v>
       </x:c>
-      <x:c r="B6" s="13" t="str">
-        <x:v>模型回答的势能差为 5.50986-7.29920 eV，均远离标准值 0.079 eV；但 alpha/beta 两个字符串字段正确，按 comparison group 取最低分后题目总分均为 0.5，压缩了答案差异。</x:v>
-      </x:c>
-      <x:c r="C6" s="14" t="str">
+      <x:c r="B6" s="89" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":0.079,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
-      <x:c r="D6" s="14" t="str">
+      <x:c r="C6" s="93" t="str">
         <x:v>potential_energy_difference：标准答案 0.079 eV，容差 ±1；ambient_pressure_phase：标准答案 alpha，精确匹配；high_pressure_phase：标准答案 beta，精确匹配。版本 linear_goal_v2。各 comparison group 取组内最低字段分，再对两组算术平均。</x:v>
       </x:c>
-      <x:c r="E6" s="14" t="str">
+      <x:c r="D6" s="93" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":7.299201259709321,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
+      <x:c r="E6" s="24" t="n">
+        <x:v>0.666667</x:v>
+      </x:c>
       <x:c r="F6" s="24" t="n">
+        <x:v>0.6666666666666666</x:v>
+      </x:c>
+      <x:c r="G6" s="93" t="str">
+        <x:v>{"answers":[{"property":"potential_energy_difference","value":5.50986,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
+      </x:c>
+      <x:c r="H6" s="24" t="n">
         <x:v>0.666667</x:v>
       </x:c>
-      <x:c r="G6" s="24" t="n">
+      <x:c r="I6" s="24" t="n">
         <x:v>0.6666666666666666</x:v>
       </x:c>
-      <x:c r="H6" s="14" t="str">
-        <x:v>{"answers":[{"property":"potential_energy_difference","value":5.50986,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
-      </x:c>
-      <x:c r="I6" s="24" t="n">
+      <x:c r="J6" s="93" t="str">
+        <x:v>{"answers":[{"property":"potential_energy_difference","value":5.51,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
+      </x:c>
+      <x:c r="K6" s="24" t="n">
         <x:v>0.666667</x:v>
       </x:c>
-      <x:c r="J6" s="24" t="n">
+      <x:c r="L6" s="24" t="n">
         <x:v>0.6666666666666666</x:v>
       </x:c>
-      <x:c r="K6" s="14" t="str">
-        <x:v>{"answers":[{"property":"potential_energy_difference","value":5.51,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
-      </x:c>
-      <x:c r="L6" s="24" t="n">
+      <x:c r="M6" s="102" t="str">
+        <x:v>{"answers":[{"property":"potential_energy_difference","value":7.17,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
+      </x:c>
+      <x:c r="N6" s="104" t="n">
         <x:v>0.666667</x:v>
       </x:c>
-      <x:c r="M6" s="69" t="n">
+      <x:c r="O6" s="104" t="n">
         <x:v>0.6666666666666666</x:v>
       </x:c>
-      <x:c r="N6" s="71" t="str">
-        <x:v>{"answers":[{"property":"potential_energy_difference","value":7.17,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
-      </x:c>
-      <x:c r="O6" s="69" t="n">
-        <x:v>0.666667</x:v>
-      </x:c>
-      <x:c r="P6" s="69" t="n">
-        <x:v>0.6666666666666666</x:v>
-      </x:c>
     </x:row>
     <x:row r="7" ht="65.1500015258789" customHeight="1">
-      <x:c r="A7" s="12" t="str">
+      <x:c r="A7" s="84" t="str">
         <x:v>property_calculation_advanced_003_hbond_count；概括：统计 DEBXIT06 晶体中一个分子参与的氢键总数。</x:v>
       </x:c>
-      <x:c r="B7" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C7" s="14" t="str">
+      <x:c r="B7" s="89" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
-      <x:c r="D7" s="14" t="str">
+      <x:c r="C7" s="93" t="str">
         <x:v>hydrogen_bond_count：标准答案 12 count；linear_goal_v2。满分：x=12。部分分：|x-12|&lt;3 按距离线性递减。0分：|x-12|≥3、单位不匹配或值无效。</x:v>
       </x:c>
-      <x:c r="E7" s="14" t="str">
+      <x:c r="D7" s="93" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
+      <x:c r="E7" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="F7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G7" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H7" s="14" t="str">
+      <x:c r="G7" s="93" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
+      <x:c r="H7" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J7" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K7" s="14" t="str">
+      <x:c r="J7" s="93" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
+      <x:c r="K7" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M7" s="69" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N7" s="71" t="str">
+      <x:c r="M7" s="102" t="str">
         <x:v>{"answer":10,"unit":"count"}</x:v>
       </x:c>
-      <x:c r="O7" s="69" t="n">
+      <x:c r="N7" s="104" t="n">
         <x:v>0.333333</x:v>
       </x:c>
-      <x:c r="P7" s="69" t="n">
+      <x:c r="O7" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="92.05000305175781" customHeight="1">
-      <x:c r="A8" s="12" t="str">
+      <x:c r="A8" s="84" t="str">
         <x:v>property_calculation_advanced_004_ir_top2_frequencies；概括：给出最低能白藜芦醇构象中 IR 强度最大的两个振动频率。</x:v>
       </x:c>
-      <x:c r="B8" s="13" t="str">
-        <x:v>题目已更新为仅取 IR 强度最大的两个频率，第三个频率存在理论与实验争议；本版采用 top2。                                   </x:v>
-      </x:c>
-      <x:c r="C8" s="14" t="str">
+      <x:c r="B8" s="89" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1208.10,"unit":"cm^-1"},{"property":"frequency_2","value":1685.56,"unit":"cm^-1"}]}</x:v>
       </x:c>
-      <x:c r="D8" s="14" t="str">
+      <x:c r="C8" s="93" t="str">
         <x:v>top_two_frequencies：两项标准答案分别为 1208.10 和 1685.56 cm^-1，各容差 ±100；采用无序最佳一一匹配，comparison group 取匹配后的最低字段分。版本 linear_goal_v2。</x:v>
       </x:c>
-      <x:c r="E8" s="14" t="str">
+      <x:c r="D8" s="93" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":435.81,"unit":"cm^-1"},{"property":"frequency_2","value":1585.74,"unit":"cm^-1"},{"property":"frequency_3","value":1592.57,"unit":"cm^-1"}]}</x:v>
       </x:c>
+      <x:c r="E8" s="24" t="n">
+        <x:v>0.0009</x:v>
+      </x:c>
       <x:c r="F8" s="24" t="n">
-        <x:v>0.0009</x:v>
-      </x:c>
-      <x:c r="G8" s="24" t="n">
         <x:v>0.000900000000000345</x:v>
       </x:c>
-      <x:c r="H8" s="14" t="str">
+      <x:c r="G8" s="93" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1585.71,"unit":"cm^-1"},{"property":"frequency_2","value":436.11,"unit":"cm^-1"},{"property":"frequency_3","value":1592.37,"unit":"cm^-1"}]}</x:v>
       </x:c>
+      <x:c r="H8" s="24" t="n">
+        <x:v>0.00075</x:v>
+      </x:c>
       <x:c r="I8" s="24" t="n">
-        <x:v>0.00075</x:v>
-      </x:c>
-      <x:c r="J8" s="24" t="n">
         <x:v>0.0007500000000004725</x:v>
       </x:c>
-      <x:c r="K8" s="14" t="str">
+      <x:c r="J8" s="93" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1584.79,"unit":"cm^-1"},{"property":"frequency_2","value":433.87,"unit":"cm^-1"},{"property":"frequency_3","value":1592.2,"unit":"cm^-1"}]}</x:v>
       </x:c>
+      <x:c r="K8" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L8" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M8" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N8" s="71" t="str">
+      <x:c r="M8" s="102" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1624.6,"unit":"cm^-1"},{"property":"frequency_2","value":1246.4,"unit":"cm^-1"},{"property":"frequency_3","value":843.1,"unit":"cm^-1"}]}</x:v>
       </x:c>
-      <x:c r="O8" s="69" t="n">
+      <x:c r="N8" s="104" t="n">
         <x:v>0.5037</x:v>
       </x:c>
-      <x:c r="P8" s="69" t="n">
+      <x:c r="O8" s="104" t="n">
         <x:v>0.5036999999999989</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="65.1500015258789" customHeight="1">
-      <x:c r="A9" s="12" t="str">
+      <x:c r="A9" s="84" t="str">
         <x:v>property_calculation_advanced_005_crystal_density；概括：估算咖啡因一水合物晶体的密度。</x:v>
       </x:c>
-      <x:c r="B9" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C9" s="14" t="str">
+      <x:c r="B9" s="89" t="str">
         <x:v>{"answer":1.44728,"unit":"g/cm^3"}</x:v>
       </x:c>
-      <x:c r="D9" s="14" t="str">
+      <x:c r="C9" s="93" t="str">
         <x:v>crystal_density：标准答案 1.44728 g/cm^3；linear_goal_v2。满分：x=1.44728。部分分：|x-1.44728|&lt;0.2 按距离线性递减。0分：|x-1.44728|≥0.2、单位不匹配或值无效。</x:v>
       </x:c>
-      <x:c r="E9" s="14" t="str">
+      <x:c r="D9" s="93" t="str">
         <x:v>{"answer":1.55,"unit":"g/cm^3"}</x:v>
       </x:c>
+      <x:c r="E9" s="24" t="n">
+        <x:v>0.4864</x:v>
+      </x:c>
       <x:c r="F9" s="24" t="n">
-        <x:v>0.4864</x:v>
-      </x:c>
-      <x:c r="G9" s="24" t="n">
         <x:v>0.2902548228400852</x:v>
       </x:c>
-      <x:c r="H9" s="14" t="str">
+      <x:c r="G9" s="93" t="str">
         <x:v>{"answer":1.56,"unit":"g/cm^3"}</x:v>
       </x:c>
+      <x:c r="H9" s="24" t="n">
+        <x:v>0.4364</x:v>
+      </x:c>
       <x:c r="I9" s="24" t="n">
-        <x:v>0.4364</x:v>
-      </x:c>
-      <x:c r="J9" s="24" t="n">
         <x:v>0.2211596926648599</x:v>
       </x:c>
-      <x:c r="K9" s="14" t="str">
+      <x:c r="J9" s="93" t="str">
         <x:v>{"answer":1.47,"unit":"g/cm^3"}</x:v>
       </x:c>
+      <x:c r="K9" s="24" t="n">
+        <x:v>0.8864</x:v>
+      </x:c>
       <x:c r="L9" s="24" t="n">
-        <x:v>0.8864</x:v>
-      </x:c>
-      <x:c r="M9" s="69" t="n">
         <x:v>0.8430158642418877</x:v>
       </x:c>
-      <x:c r="N9" s="71" t="str">
+      <x:c r="M9" s="102" t="str">
         <x:v>{"answer":1.28,"unit":"g/cm^3"}</x:v>
       </x:c>
-      <x:c r="O9" s="69" t="n">
+      <x:c r="N9" s="104" t="n">
         <x:v>0.1636</x:v>
       </x:c>
-      <x:c r="P9" s="69" t="n">
+      <x:c r="O9" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="50.900001525878906" customHeight="1">
-      <x:c r="A10" s="12" t="str">
+      <x:c r="A10" s="84" t="str">
         <x:v>property_calculation_advanced_006_cocrystal_ratio；概括：确定大麻酚与四甲基吡嗪在最终共晶中的摩尔比。</x:v>
       </x:c>
-      <x:c r="B10" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C10" s="14" t="str">
+      <x:c r="B10" s="89" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
-      <x:c r="D10" s="14" t="str">
+      <x:c r="C10" s="93" t="str">
         <x:v>cocrystal_ratio：标准答案 1:1；版本 linear_goal_v2。精确匹配得 1 分；1:2 或 2:1 得 0.5 分；其他结果得 0 分。</x:v>
       </x:c>
-      <x:c r="E10" s="14" t="str">
+      <x:c r="D10" s="93" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
+      <x:c r="E10" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="F10" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G10" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H10" s="14" t="str">
+      <x:c r="G10" s="93" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
+      <x:c r="H10" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="I10" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="J10" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="K10" s="14" t="str">
+      <x:c r="J10" s="93" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
+      <x:c r="K10" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L10" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M10" s="69" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N10" s="71" t="str">
+      <x:c r="M10" s="102" t="str">
         <x:v>{"answer":"1:2"}</x:v>
       </x:c>
-      <x:c r="O10" s="69" t="n">
+      <x:c r="N10" s="104" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="P10" s="69" t="n">
+      <x:c r="O10" s="104" t="n">
         <x:v>0.5</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="68.05000305175781" customHeight="1">
-      <x:c r="A11" s="12" t="str">
+      <x:c r="A11" s="84" t="str">
         <x:v>property_calculation_advanced_007_polymorph_free_energy_crossover；概括：判断 Radiprodil FormA/FormC 在 0 K 的低自由能晶型及交叉温度。</x:v>
       </x:c>
-      <x:c r="B11" s="13" t="str">
-        <x:v>不同模型给出的低能晶型与交叉温度差异很大，但按题目字段最低分聚合后多数组合均为 0，完全掩盖了答案差异。两个字段应该分开评分</x:v>
-      </x:c>
-      <x:c r="C11" s="14" t="str">
+      <x:c r="B11" s="89" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormC"},{"property":"crossover_temperature","value":343.15,"unit":"K"}]}</x:v>
       </x:c>
-      <x:c r="D11" s="14" t="str">
+      <x:c r="C11" s="93" t="str">
         <x:v>lower_free_energy_at_0k：标准答案 FormC，精确匹配；crossover_temperature：标准答案 343.15 K，容差 ±200。版本 linear_goal_v2。题目分取全部字段中的最低值。</x:v>
       </x:c>
-      <x:c r="E11" s="14" t="str">
+      <x:c r="D11" s="93" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":3016,"unit":"K"}]}</x:v>
       </x:c>
+      <x:c r="E11" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F11" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G11" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H11" s="14" t="str">
+      <x:c r="G11" s="93" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormC"},{"property":"crossover_temperature","value":943,"unit":"K"}]}</x:v>
+      </x:c>
+      <x:c r="H11" s="24" t="n">
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="I11" s="24" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="J11" s="24" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="K11" s="14" t="str">
+      <x:c r="J11" s="93" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":428.5,"unit":"K"}]}</x:v>
       </x:c>
+      <x:c r="K11" s="24" t="n">
+        <x:v>0.286625</x:v>
+      </x:c>
       <x:c r="L11" s="24" t="n">
-        <x:v>0.286625</x:v>
-      </x:c>
-      <x:c r="M11" s="69" t="n">
         <x:v>0.07324999999999987</x:v>
       </x:c>
-      <x:c r="N11" s="71" t="str">
+      <x:c r="M11" s="102" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":300,"unit":"K"}]}</x:v>
       </x:c>
-      <x:c r="O11" s="69" t="n">
+      <x:c r="N11" s="104" t="n">
         <x:v>0.392125</x:v>
       </x:c>
-      <x:c r="P11" s="69" t="n">
+      <x:c r="O11" s="104" t="n">
         <x:v>0.2842500000000001</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="68.05000305175781" customHeight="1">
-      <x:c r="A12" s="12" t="str">
+      <x:c r="A12" s="84" t="str">
         <x:v>property_calculation_advanced_008_interaction_binding_energy；概括：计算指定二聚体的相互作用能和结合能并保留符号。</x:v>
       </x:c>
-      <x:c r="B12" s="13" t="str">
-        <x:v>两个字段也应该分开评分</x:v>
-      </x:c>
-      <x:c r="C12" s="14" t="str">
+      <x:c r="B12" s="89" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-69.04,"unit":"kcal/mol"},{"property":"binding_energy","value":-58.15,"unit":"kcal/mol"}]}</x:v>
       </x:c>
-      <x:c r="D12" s="14" t="str">
+      <x:c r="C12" s="93" t="str">
         <x:v>interaction_energy 与 binding_energy：标准答案分别为 -69.04 和 -58.15 kcal/mol；先取绝对值再按 ±20 线性评分。版本 linear_goal_v2。题目分取两字段最低值。</x:v>
       </x:c>
-      <x:c r="E12" s="14" t="str">
+      <x:c r="D12" s="93" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.4733,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.3678,"unit":"kcal/mol"}]}</x:v>
       </x:c>
+      <x:c r="E12" s="24" t="n">
+        <x:v>0.933723</x:v>
+      </x:c>
       <x:c r="F12" s="24" t="n">
-        <x:v>0.933723</x:v>
-      </x:c>
-      <x:c r="G12" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H12" s="14" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G12" s="93" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.47,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.38,"unit":"kcal/mol"}]}</x:v>
       </x:c>
+      <x:c r="H12" s="24" t="n">
+        <x:v>0.9335</x:v>
+      </x:c>
       <x:c r="I12" s="24" t="n">
-        <x:v>0.9335</x:v>
-      </x:c>
-      <x:c r="J12" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K12" s="14" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J12" s="93" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.45,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.37,"unit":"kcal/mol"}]}</x:v>
       </x:c>
+      <x:c r="K12" s="24" t="n">
+        <x:v>0.93425</x:v>
+      </x:c>
       <x:c r="L12" s="24" t="n">
-        <x:v>0.93425</x:v>
-      </x:c>
-      <x:c r="M12" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N12" s="71" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M12" s="102" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.49,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.38,"unit":"kcal/mol"}]}</x:v>
       </x:c>
-      <x:c r="O12" s="69" t="n">
+      <x:c r="N12" s="104" t="n">
         <x:v>0.933</x:v>
       </x:c>
-      <x:c r="P12" s="69" t="n">
+      <x:c r="O12" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="65.1500015258789" customHeight="1">
-      <x:c r="A13" s="12" t="str">
+      <x:c r="A13" s="84" t="str">
         <x:v>property_calculation_advanced_009_homo_lumo_gap；概括：计算指定分子的 HOMO-LUMO 能隙。</x:v>
       </x:c>
-      <x:c r="B13" s="13" t="str">
-        <x:v>四组都拿不到分</x:v>
-      </x:c>
-      <x:c r="C13" s="14" t="str">
+      <x:c r="B13" s="89" t="str">
         <x:v>{"answer":7.26,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="D13" s="14" t="str">
+      <x:c r="C13" s="93" t="str">
         <x:v>homo_lumo_gap：标准答案 7.26 eV；linear_goal_v2。满分：x=7.26。部分分：|x-7.26|&lt;2 按距离线性递减。0分：|x-7.26|≥2、单位不匹配或值无效。</x:v>
       </x:c>
-      <x:c r="E13" s="14" t="str">
+      <x:c r="D13" s="93" t="str">
         <x:v>{"answer":3.558797467914,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="E13" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F13" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G13" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H13" s="14" t="str">
+      <x:c r="G13" s="93" t="str">
         <x:v>{"answer":3.559175368755,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="H13" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="I13" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J13" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K13" s="14" t="str">
+      <x:c r="J13" s="93" t="str">
         <x:v>{"answer":3.5845,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="K13" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L13" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M13" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N13" s="71" t="str">
+      <x:c r="M13" s="102" t="str">
         <x:v>{"answer":3.584,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="O13" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P13" s="69" t="n">
+      <x:c r="N13" s="104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O13" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="68.05000305175781" customHeight="1">
-      <x:c r="A14" s="12" t="str">
+      <x:c r="A14" s="84" t="str">
         <x:v>property_calculation_advanced_010_hbond_distances；概括：计算尿素-磷酸相互作用单元的 O-H 键长与 H...O 接触距离。</x:v>
       </x:c>
-      <x:c r="B14" s="13" t="str">
-        <x:v>两个字段也应该分开评分</x:v>
-      </x:c>
-      <x:c r="C14" s="14" t="str">
+      <x:c r="B14" s="89" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.029,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.485,"unit":"angstrom"}]}</x:v>
       </x:c>
-      <x:c r="D14" s="14" t="str">
+      <x:c r="C14" s="93" t="str">
         <x:v>oh_bond_distance 与 h_o_contact_distance：标准答案分别为 1.029 和 1.485 angstrom；先取绝对值再按 ±0.3 线性评分。版本 linear_goal_v2。题目分取两字段最低值。</x:v>
       </x:c>
-      <x:c r="E14" s="14" t="str">
+      <x:c r="D14" s="93" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
+      <x:c r="E14" s="24" t="n">
+        <x:v>0.776667</x:v>
+      </x:c>
       <x:c r="F14" s="24" t="n">
+        <x:v>0.6650000000000003</x:v>
+      </x:c>
+      <x:c r="G14" s="93" t="str">
+        <x:v>{"answers":[{"property":"oh_bond_distance","value":1.001520301,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.594671850,"unit":"angstrom"}]}</x:v>
+      </x:c>
+      <x:c r="H14" s="24" t="n">
+        <x:v>0.771414</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="n">
+        <x:v>0.6571211275000007</x:v>
+      </x:c>
+      <x:c r="J14" s="93" t="str">
+        <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
+      </x:c>
+      <x:c r="K14" s="24" t="n">
         <x:v>0.776667</x:v>
       </x:c>
-      <x:c r="G14" s="24" t="n">
+      <x:c r="L14" s="24" t="n">
         <x:v>0.6650000000000003</x:v>
       </x:c>
-      <x:c r="H14" s="14" t="str">
-        <x:v>{"answers":[{"property":"oh_bond_distance","value":1.001520301,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.594671850,"unit":"angstrom"}]}</x:v>
-      </x:c>
-      <x:c r="I14" s="24" t="n">
-        <x:v>0.771414</x:v>
-      </x:c>
-      <x:c r="J14" s="24" t="n">
-        <x:v>0.6571211275000007</x:v>
-      </x:c>
-      <x:c r="K14" s="14" t="str">
+      <x:c r="M14" s="102" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
-      <x:c r="L14" s="24" t="n">
+      <x:c r="N14" s="104" t="n">
         <x:v>0.776667</x:v>
       </x:c>
-      <x:c r="M14" s="69" t="n">
+      <x:c r="O14" s="104" t="n">
         <x:v>0.6650000000000003</x:v>
       </x:c>
-      <x:c r="N14" s="71" t="str">
-        <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
-      </x:c>
-      <x:c r="O14" s="69" t="n">
-        <x:v>0.776667</x:v>
-      </x:c>
-      <x:c r="P14" s="69" t="n">
-        <x:v>0.6650000000000003</x:v>
-      </x:c>
     </x:row>
     <x:row r="15" ht="65.1500015258789" customHeight="1">
-      <x:c r="A15" s="12" t="str">
+      <x:c r="A15" s="84" t="str">
         <x:v>property_calculation_advanced_011_accessible_pore_volume_ratio；概括：计算 NOGCOE 晶胞的可达体积与不可达体积之比。</x:v>
       </x:c>
-      <x:c r="B15" s="13" t="str">
-        <x:v>四组都拿不到分</x:v>
-      </x:c>
-      <x:c r="C15" s="14" t="str">
+      <x:c r="B15" s="89" t="str">
         <x:v>{"answer":1.713,"unit":"ratio"}</x:v>
       </x:c>
-      <x:c r="D15" s="14" t="str">
+      <x:c r="C15" s="93" t="str">
         <x:v>accessible_to_inaccessible_volume_ratio：标准答案 1.713 ratio；linear_goal_v2。满分：x=1.713。部分分：|x-1.713|&lt;0.5 按距离线性递减。0分：|x-1.713|≥0.5、单位不匹配或值无效。</x:v>
       </x:c>
-      <x:c r="E15" s="14" t="str">
+      <x:c r="D15" s="93" t="str">
         <x:v>{"answer":0.0443,"unit":"ratio"}</x:v>
       </x:c>
+      <x:c r="E15" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F15" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G15" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H15" s="14" t="str">
+      <x:c r="G15" s="93" t="str">
         <x:v>{"answer":0.07236,"unit":"ratio"}</x:v>
       </x:c>
+      <x:c r="H15" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="I15" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J15" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K15" s="14" t="str">
+      <x:c r="J15" s="93" t="str">
         <x:v>{"answer":0.076,"unit":"ratio"}</x:v>
       </x:c>
+      <x:c r="K15" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L15" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M15" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N15" s="71" t="str">
+      <x:c r="M15" s="102" t="str">
         <x:v>{"answer":0.0724,"unit":"ratio"}</x:v>
       </x:c>
-      <x:c r="O15" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P15" s="69" t="n">
+      <x:c r="N15" s="104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O15" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="65.1500015258789" customHeight="1">
-      <x:c r="A16" s="12" t="str">
+      <x:c r="A16" s="84" t="str">
         <x:v>property_calculation_advanced_012_carboxyl_hydrogen_distance；概括：计算指定二羧酸最低能构象中两个羧酸氢的距离。</x:v>
       </x:c>
-      <x:c r="B16" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C16" s="14" t="str">
+      <x:c r="B16" s="89" t="str">
         <x:v>{"answer":2.521,"unit":"angstrom"}</x:v>
       </x:c>
-      <x:c r="D16" s="14" t="str">
+      <x:c r="C16" s="93" t="str">
         <x:v>carboxyl_hydrogen_distance：标准答案 2.521 angstrom；linear_goal_v2。满分：x=2.521。部分分：|x-2.521|&lt;0.5 按距离线性递减。0分：|x-2.521|≥0.5、单位不匹配或值无效。</x:v>
       </x:c>
-      <x:c r="E16" s="14" t="str">
+      <x:c r="D16" s="93" t="str">
         <x:v>{"answer":2.5212,"unit":"angstrom"}</x:v>
       </x:c>
+      <x:c r="E16" s="24" t="n">
+        <x:v>0.9996</x:v>
+      </x:c>
       <x:c r="F16" s="24" t="n">
-        <x:v>0.9996</x:v>
-      </x:c>
-      <x:c r="G16" s="24" t="n">
         <x:v>0.9990000000000001</x:v>
       </x:c>
-      <x:c r="H16" s="14" t="str">
+      <x:c r="G16" s="93" t="str">
         <x:v>{"answer":2.5183,"unit":"angstrom"}</x:v>
       </x:c>
+      <x:c r="H16" s="24" t="n">
+        <x:v>0.9946</x:v>
+      </x:c>
       <x:c r="I16" s="24" t="n">
-        <x:v>0.9946</x:v>
-      </x:c>
-      <x:c r="J16" s="24" t="n">
         <x:v>0.9865000000000004</x:v>
       </x:c>
-      <x:c r="K16" s="14" t="str">
+      <x:c r="J16" s="93" t="str">
         <x:v>{"answer":2.52,"unit":"angstrom"}</x:v>
       </x:c>
+      <x:c r="K16" s="24" t="n">
+        <x:v>0.998</x:v>
+      </x:c>
       <x:c r="L16" s="24" t="n">
-        <x:v>0.998</x:v>
-      </x:c>
-      <x:c r="M16" s="69" t="n">
         <x:v>0.9950000000000006</x:v>
       </x:c>
-      <x:c r="N16" s="71" t="str">
+      <x:c r="M16" s="102" t="str">
         <x:v>{"answer":2.7043,"unit":"angstrom"}</x:v>
       </x:c>
-      <x:c r="O16" s="69" t="n">
+      <x:c r="N16" s="104" t="n">
         <x:v>0.6334</x:v>
       </x:c>
-      <x:c r="P16" s="69" t="n">
+      <x:c r="O16" s="104" t="n">
         <x:v>0.08349999999999991</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="65.1500015258789" customHeight="1">
-      <x:c r="A17" s="12" t="str">
+      <x:c r="A17" s="84" t="str">
         <x:v>property_calculation_advanced_013_halogen_bond_energy；概括：计算 FI...NH3 卤键复合物的相互作用能并保留符号。</x:v>
       </x:c>
-      <x:c r="B17" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C17" s="14" t="str">
+      <x:c r="B17" s="89" t="str">
         <x:v>{"answer":-17.11,"unit":"kcal/mol"}</x:v>
       </x:c>
-      <x:c r="D17" s="14" t="str">
+      <x:c r="C17" s="93" t="str">
         <x:v>halogen_bond_interaction_energy：标准答案 -17.11 kcal/mol；先取绝对值再按 ±5 线性评分。版本 linear_goal_v2。0分：绝对值误差≥5、单位不匹配或值无效。</x:v>
       </x:c>
-      <x:c r="E17" s="14" t="str">
+      <x:c r="D17" s="93" t="str">
         <x:v>{"answer":-17.11,"unit":"kcal/mol"}</x:v>
       </x:c>
+      <x:c r="E17" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="F17" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G17" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H17" s="14" t="str">
+      <x:c r="G17" s="93" t="str">
         <x:v>{"answer":-19.17,"unit":"kcal/mol"}</x:v>
       </x:c>
+      <x:c r="H17" s="24" t="n">
+        <x:v>0.588</x:v>
+      </x:c>
       <x:c r="I17" s="24" t="n">
-        <x:v>0.588</x:v>
-      </x:c>
-      <x:c r="J17" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K17" s="14" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J17" s="93" t="str">
         <x:v>{"answer":-15.5969,"unit":"kcal/mol"}</x:v>
       </x:c>
+      <x:c r="K17" s="24" t="n">
+        <x:v>0.69738</x:v>
+      </x:c>
       <x:c r="L17" s="24" t="n">
-        <x:v>0.69738</x:v>
-      </x:c>
-      <x:c r="M17" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N17" s="71" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M17" s="102" t="str">
         <x:v>{"answer":-16.5,"unit":"kcal/mol"}</x:v>
       </x:c>
-      <x:c r="O17" s="69" t="n">
+      <x:c r="N17" s="104" t="n">
         <x:v>0.878</x:v>
       </x:c>
-      <x:c r="P17" s="69" t="n">
+      <x:c r="O17" s="104" t="n">
         <x:v>0.39000000000000057</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="50.900001525878906" customHeight="1">
-      <x:c r="A18" s="12" t="str">
+      <x:c r="A18" s="84" t="str">
         <x:v>property_calculation_advanced_014_bay069_pka；概括：计算 BAY-069 分子的 pKa。</x:v>
       </x:c>
-      <x:c r="B18" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C18" s="14" t="str">
+      <x:c r="B18" s="89" t="str">
         <x:v>{"answer":5.7,"unit":"pKa"}</x:v>
       </x:c>
-      <x:c r="D18" s="14" t="str">
+      <x:c r="C18" s="93" t="str">
         <x:v>pka：标准答案 5.7 pKa；linear_goal_v2。满分：x=5.7。部分分：|x-5.7|&lt;2 按距离线性递减。0分：|x-5.7|≥2、单位不匹配或值无效。</x:v>
       </x:c>
-      <x:c r="E18" s="14" t="str">
+      <x:c r="D18" s="93" t="str">
         <x:v>{"answer":5.0,"unit":"pKa"}</x:v>
       </x:c>
+      <x:c r="E18" s="24" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
       <x:c r="F18" s="24" t="n">
-        <x:v>0.65</x:v>
-      </x:c>
-      <x:c r="G18" s="24" t="n">
         <x:v>0.6499999999999999</x:v>
       </x:c>
-      <x:c r="H18" s="14" t="str">
+      <x:c r="G18" s="93" t="str">
         <x:v>{"answer":6.33,"unit":"pKa"}</x:v>
+      </x:c>
+      <x:c r="H18" s="24" t="n">
+        <x:v>0.685</x:v>
       </x:c>
       <x:c r="I18" s="24" t="n">
         <x:v>0.685</x:v>
       </x:c>
-      <x:c r="J18" s="24" t="n">
-        <x:v>0.685</x:v>
-      </x:c>
-      <x:c r="K18" s="14" t="str">
+      <x:c r="J18" s="93" t="str">
         <x:v>{"answer":5.7,"unit":"pKa"}</x:v>
       </x:c>
+      <x:c r="K18" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L18" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M18" s="69" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N18" s="71" t="str">
+      <x:c r="M18" s="102" t="str">
         <x:v>{"answer":6.8,"unit":"pKa"}</x:v>
       </x:c>
-      <x:c r="O18" s="69" t="n">
+      <x:c r="N18" s="104" t="n">
         <x:v>0.45</x:v>
       </x:c>
-      <x:c r="P18" s="69" t="n">
+      <x:c r="O18" s="104" t="n">
         <x:v>0.4500000000000002</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="65.1500015258789" customHeight="1">
-      <x:c r="A19" s="12" t="str">
+      <x:c r="A19" s="84" t="str">
         <x:v>property_calculation_advanced_015_formaldehyde_socme；概括：计算气相甲醛 T1-S0 自旋轨道耦合矩阵元的大小。</x:v>
       </x:c>
-      <x:c r="B19" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C19" s="14" t="str">
+      <x:c r="B19" s="89" t="str">
         <x:v>{"answer":0.00734,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="D19" s="14" t="str">
+      <x:c r="C19" s="93" t="str">
         <x:v>spin_orbit_coupling_matrix_element：标准答案 0.00734 eV；对 x 与标准答案分别取 log10，在 log10 空间按 ±1 线性评分。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
       </x:c>
-      <x:c r="E19" s="14" t="str">
+      <x:c r="D19" s="93" t="str">
         <x:v>{"answer":0.00485,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="E19" s="24" t="n">
+        <x:v>0.820046</x:v>
+      </x:c>
       <x:c r="F19" s="24" t="n">
-        <x:v>0.820046</x:v>
-      </x:c>
-      <x:c r="G19" s="24" t="n">
         <x:v>0.8200456786861929</x:v>
       </x:c>
-      <x:c r="H19" s="14" t="str">
+      <x:c r="G19" s="93" t="str">
         <x:v>{"answer":0.0035,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="H19" s="24" t="n">
+        <x:v>0.678372</x:v>
+      </x:c>
       <x:c r="I19" s="24" t="n">
-        <x:v>0.678372</x:v>
-      </x:c>
-      <x:c r="J19" s="24" t="n">
         <x:v>0.6783719844342051</x:v>
       </x:c>
-      <x:c r="K19" s="14" t="str">
+      <x:c r="J19" s="93" t="str">
         <x:v>{"answer":0.0,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="K19" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="L19" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="M19" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N19" s="71" t="str">
+      <x:c r="M19" s="102" t="str">
         <x:v>{"answer":0.01,"unit":"eV"}</x:v>
       </x:c>
-      <x:c r="O19" s="69" t="n">
+      <x:c r="N19" s="104" t="n">
         <x:v>0.865696</x:v>
       </x:c>
-      <x:c r="P19" s="69" t="n">
+      <x:c r="O19" s="104" t="n">
         <x:v>0.8656960599160706</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="65.1500015258789" customHeight="1">
-      <x:c r="A20" s="12" t="str">
+      <x:c r="A20" s="84" t="str">
         <x:v>property_calculation_advanced_016_anthracene_isc_rate；概括：计算气相蒽在 77 K 的 S1 系间窜越速率常数。</x:v>
       </x:c>
-      <x:c r="B20" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C20" s="14" t="str">
+      <x:c r="B20" s="89" t="str">
         <x:v>{"answer":117000000,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="D20" s="14" t="str">
+      <x:c r="C20" s="93" t="str">
         <x:v>intersystem_crossing_rate：标准答案 117000000 s^-1；对 x 与标准答案分别取 log10，在 log10 空间按 ±3 线性评分。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
       </x:c>
-      <x:c r="E20" s="14" t="str">
+      <x:c r="D20" s="93" t="str">
         <x:v>{"answer":1.2e8,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="E20" s="24" t="n">
+        <x:v>0.996335</x:v>
+      </x:c>
       <x:c r="F20" s="24" t="n">
-        <x:v>0.996335</x:v>
-      </x:c>
-      <x:c r="G20" s="24" t="n">
         <x:v>0.9945023078492685</x:v>
       </x:c>
-      <x:c r="H20" s="14" t="str">
+      <x:c r="G20" s="93" t="str">
         <x:v>{"answer":1.45e8,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="H20" s="24" t="n">
+        <x:v>0.968939</x:v>
+      </x:c>
       <x:c r="I20" s="24" t="n">
-        <x:v>0.968939</x:v>
-      </x:c>
-      <x:c r="J20" s="24" t="n">
         <x:v>0.9534089297555939</x:v>
       </x:c>
-      <x:c r="K20" s="14" t="str">
+      <x:c r="J20" s="93" t="str">
         <x:v>{"answer":1e6,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="K20" s="24" t="n">
+        <x:v>0.310605</x:v>
+      </x:c>
       <x:c r="L20" s="24" t="n">
-        <x:v>0.310605</x:v>
-      </x:c>
-      <x:c r="M20" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="N20" s="71" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="M20" s="102" t="str">
         <x:v>{"answer":100000,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="O20" s="69" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P20" s="69" t="n">
+      <x:c r="N20" s="104" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O20" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="79.4000015258789" customHeight="1">
-      <x:c r="A21" s="12" t="str">
+      <x:c r="A21" s="84" t="str">
         <x:v>property_calculation_advanced_017_biacetyl_phosphorescence_rate；概括：计算乙醇隐式溶剂中联乙酰在 298 K 的磷光速率常数。</x:v>
       </x:c>
-      <x:c r="B21" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C21" s="14" t="str">
+      <x:c r="B21" s="89" t="str">
         <x:v>{"answer":98,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="D21" s="14" t="str">
+      <x:c r="C21" s="93" t="str">
         <x:v>phosphorescence_rate：标准答案 98 s^-1；对 x 与标准答案分别取 log10，在 log10 空间下侧容差 2、上侧容差 3，按线性距离递减。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
       </x:c>
-      <x:c r="E21" s="14" t="str">
+      <x:c r="D21" s="93" t="str">
         <x:v>{"answer":91.92785,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="E21" s="24" t="n">
+        <x:v>0.986111</x:v>
+      </x:c>
       <x:c r="F21" s="24" t="n">
-        <x:v>0.986111</x:v>
-      </x:c>
-      <x:c r="G21" s="24" t="n">
         <x:v>0.9861105136520333</x:v>
       </x:c>
-      <x:c r="H21" s="14" t="str">
+      <x:c r="G21" s="93" t="str">
         <x:v>{"answer":100.0,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="H21" s="24" t="n">
+        <x:v>0.997075</x:v>
+      </x:c>
       <x:c r="I21" s="24" t="n">
+        <x:v>0.9956130378462474</x:v>
+      </x:c>
+      <x:c r="J21" s="93" t="str">
+        <x:v>{"answer":100,"unit":"s^-1"}</x:v>
+      </x:c>
+      <x:c r="K21" s="24" t="n">
         <x:v>0.997075</x:v>
       </x:c>
-      <x:c r="J21" s="24" t="n">
+      <x:c r="L21" s="24" t="n">
         <x:v>0.9956130378462474</x:v>
       </x:c>
-      <x:c r="K21" s="14" t="str">
-        <x:v>{"answer":100,"unit":"s^-1"}</x:v>
-      </x:c>
-      <x:c r="L21" s="24" t="n">
-        <x:v>0.997075</x:v>
-      </x:c>
-      <x:c r="M21" s="69" t="n">
-        <x:v>0.9956130378462474</x:v>
-      </x:c>
-      <x:c r="N21" s="71" t="str">
+      <x:c r="M21" s="102" t="str">
         <x:v>{"answer":16.9,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="O21" s="69" t="n">
+      <x:c r="N21" s="104" t="n">
         <x:v>0.61833</x:v>
       </x:c>
-      <x:c r="P21" s="69" t="n">
+      <x:c r="O21" s="104" t="n">
         <x:v>0.6183303144605893</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="65.1500015258789" customHeight="1">
-      <x:c r="A22" s="12" t="str">
+      <x:c r="A22" s="84" t="str">
         <x:v>property_calculation_advanced_018_anthracene_ht_contribution；概括：计算气相蒽在 77 K 的 Herzberg-Teller 项对 S1-T1 系间窜越速率的贡献比例。</x:v>
       </x:c>
-      <x:c r="B22" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C22" s="14" t="str">
+      <x:c r="B22" s="89" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
-      <x:c r="D22" s="14" t="str">
+      <x:c r="C22" s="93" t="str">
         <x:v>herzberg_teller_contribution：标准答案 100 percent；linear_goal_v2。下侧容差 10、上侧容差 1，按距离线性递减；0分：低于 90 或高于 101、单位不匹配或值无效。</x:v>
       </x:c>
-      <x:c r="E22" s="14" t="str">
+      <x:c r="D22" s="93" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
+      <x:c r="E22" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="F22" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="G22" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="H22" s="14" t="str">
+      <x:c r="G22" s="93" t="str">
         <x:v>{"answer":70,"unit":"percent"}</x:v>
       </x:c>
+      <x:c r="H22" s="24" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="I22" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J22" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K22" s="14" t="str">
+      <x:c r="J22" s="93" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
+      <x:c r="K22" s="24" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="L22" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="M22" s="69" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="N22" s="71" t="str">
+      <x:c r="M22" s="102" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
-      <x:c r="O22" s="69" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="P22" s="69" t="n">
+      <x:c r="N22" s="104" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="O22" s="104" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="79.4000015258789" customHeight="1">
-      <x:c r="A23" s="12" t="str">
+      <x:c r="A23" s="84" t="str">
         <x:v>property_calculation_advanced_019_acetophenone_isc_rate；概括：计算气相苯乙酮在 77 K 含 Herzberg-Teller 效应的 S1-T1 系间窜越速率。</x:v>
       </x:c>
-      <x:c r="B23" s="13" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C23" s="14" t="str">
+      <x:c r="B23" s="89" t="str">
         <x:v>{"answer":28400000000,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="D23" s="14" t="str">
+      <x:c r="C23" s="93" t="str">
         <x:v>intersystem_crossing_rate：标准答案 28400000000 s^-1；对 x 与标准答案分别取 log10，在 log10 空间按 ±3 线性评分。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
       </x:c>
-      <x:c r="E23" s="14" t="str">
+      <x:c r="D23" s="93" t="str">
         <x:v>{"answer":2.38e10,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="E23" s="24" t="n">
+        <x:v>0.97442</x:v>
+      </x:c>
       <x:c r="F23" s="24" t="n">
-        <x:v>0.97442</x:v>
-      </x:c>
-      <x:c r="G23" s="24" t="n">
         <x:v>0.9616293085047376</x:v>
       </x:c>
-      <x:c r="H23" s="14" t="str">
+      <x:c r="G23" s="93" t="str">
         <x:v>{"answer":1.6e8,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="H23" s="24" t="n">
+        <x:v>0.250267</x:v>
+      </x:c>
       <x:c r="I23" s="24" t="n">
-        <x:v>0.250267</x:v>
-      </x:c>
-      <x:c r="J23" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K23" s="14" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J23" s="93" t="str">
         <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="K23" s="24" t="n">
+        <x:v>0.848894</x:v>
+      </x:c>
       <x:c r="L23" s="24" t="n">
+        <x:v>0.7733408299764815</x:v>
+      </x:c>
+      <x:c r="M23" s="102" t="str">
+        <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
+      </x:c>
+      <x:c r="N23" s="104" t="n">
         <x:v>0.848894</x:v>
       </x:c>
-      <x:c r="M23" s="69" t="n">
+      <x:c r="O23" s="104" t="n">
         <x:v>0.7733408299764815</x:v>
       </x:c>
-      <x:c r="N23" s="71" t="str">
-        <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
-      </x:c>
-      <x:c r="O23" s="69" t="n">
-        <x:v>0.848894</x:v>
-      </x:c>
-      <x:c r="P23" s="69" t="n">
-        <x:v>0.7733408299764815</x:v>
-      </x:c>
     </x:row>
     <x:row r="24" ht="65.1500015258789" customHeight="1">
-      <x:c r="A24" s="15" t="str">
+      <x:c r="A24" s="85" t="str">
         <x:v>property_calculation_advanced_020_azulene_internal_conversion_rate；概括：计算甲醇隐式溶剂中薁在 298.15 K 的 S1-S0 内转换速率。</x:v>
       </x:c>
-      <x:c r="B24" s="16" t="str">
-        <x:v>合理</x:v>
-      </x:c>
-      <x:c r="C24" s="17" t="str">
+      <x:c r="B24" s="90" t="str">
         <x:v>{"answer":382000000,"unit":"s^-1"}</x:v>
       </x:c>
-      <x:c r="D24" s="17" t="str">
+      <x:c r="C24" s="94" t="str">
         <x:v>internal_conversion_rate：标准答案 382000000 s^-1；对 x 与标准答案分别取 log10，在 log10 空间按 ±3 线性评分。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
       </x:c>
-      <x:c r="E24" s="17" t="str">
+      <x:c r="D24" s="94" t="str">
         <x:v>{"answer":1e12,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="E24" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="F24" s="25" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="G24" s="25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H24" s="17" t="str">
+      <x:c r="G24" s="94" t="str">
         <x:v>{"answer":9.4e11,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="H24" s="25" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="I24" s="25" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="J24" s="25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="K24" s="18" t="str">
+      <x:c r="J24" s="98" t="str">
         <x:v>{"answer":1.0e9,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="K24" s="25" t="n">
+        <x:v>0.860688</x:v>
+      </x:c>
       <x:c r="L24" s="25" t="n">
-        <x:v>0.860688</x:v>
-      </x:c>
-      <x:c r="M24" s="74" t="n">
         <x:v>0.7910316814558547</x:v>
       </x:c>
-      <x:c r="N24" s="75"/>
-      <x:c r="O24" s="74" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="P24" s="74" t="n">
+      <x:c r="M24" s="57"/>
+      <x:c r="N24" s="43" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="O24" s="43" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="28" customHeight="1">
-      <x:c r="A25" s="19" t="str">
+      <x:c r="A25" s="86" t="str">
         <x:v>各实验组平均分（未评分项记0分）</x:v>
       </x:c>
-      <x:c r="B25" s="20"/>
-      <x:c r="C25" s="20"/>
-      <x:c r="D25" s="20"/>
-      <x:c r="E25" s="21" t="str">
+      <x:c r="B25" s="91"/>
+      <x:c r="C25" s="91"/>
+      <x:c r="D25" s="96" t="str">
         <x:v>平均分</x:v>
       </x:c>
+      <x:c r="E25" s="26" t="n">
+        <x:v>0.663653</x:v>
+      </x:c>
       <x:c r="F25" s="26" t="n">
-        <x:v>0.663653</x:v>
-      </x:c>
-      <x:c r="G25" s="26" t="n">
         <x:v>0.6005921419161993</x:v>
       </x:c>
-      <x:c r="H25" s="22" t="str">
+      <x:c r="G25" s="97" t="str">
         <x:v>平均分</x:v>
       </x:c>
+      <x:c r="H25" s="26" t="n">
+        <x:v>0.523549</x:v>
+      </x:c>
       <x:c r="I25" s="26" t="n">
-        <x:v>0.523549</x:v>
-      </x:c>
-      <x:c r="J25" s="26" t="n">
         <x:v>0.41722957194337873</x:v>
       </x:c>
-      <x:c r="K25" s="21" t="str">
+      <x:c r="J25" s="96" t="str">
         <x:v>平均分</x:v>
       </x:c>
+      <x:c r="K25" s="26" t="n">
+        <x:v>0.662272</x:v>
+      </x:c>
       <x:c r="L25" s="26" t="n">
-        <x:v>0.662272</x:v>
-      </x:c>
-      <x:c r="M25" s="76" t="n">
         <x:v>0.5390332060156069</x:v>
       </x:c>
-      <x:c r="N25" s="77" t="str">
+      <x:c r="M25" s="61" t="str">
         <x:v>平均分</x:v>
       </x:c>
-      <x:c r="O25" s="76" t="n">
+      <x:c r="N25" s="47" t="n">
         <x:v>0.515411</x:v>
       </x:c>
-      <x:c r="P25" s="76" t="n">
+      <x:c r="O25" s="47" t="n">
         <x:v>0.37407439154474037</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
fix: remove scoring notes from score workbooks
</commit_message>
<xml_diff>
--- a/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.9.3-rescored.xlsx
+++ b/outputs/01a0b000-cf04-7f00-a568-1f20935b5dd8/vgb-property-calculation-advanced-v0.9.3-rescored.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="R785ec70e719f4c04"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="工作表 1" sheetId="1" r:id="Rd5303dbba5ae4aa1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -960,18 +960,18 @@
   <x:cols>
     <x:col min="1" max="1" width="23.171899795532227" style="1" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="26.171899795532227" style="1" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="29.851600646972656" style="1" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="19.351600646972656" style="1" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="12.35159969329834" style="1" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="18" style="1" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="13.5" style="1" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="17" style="1" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="12" style="1" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="17.5" style="1" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="19.351600646972656" style="1" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12.35159969329834" style="1" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" style="1" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="13.5" style="1" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="17" style="1" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="12" style="1" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="17.5" style="1" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="16.351600646972656" style="1" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="16.351600646972656" style="1" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="16.351600646972656" style="1" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="17.5" style="1" hidden="0" customWidth="1"/>
     <x:col min="13" max="16384" width="16.351600646972656" style="1" customWidth="1"/>
-    <x:col min="13" max="13" width="17.5" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="16.351600646972656" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="16.351600646972656" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="16.351600646972656" hidden="0" customWidth="1"/>
     <x:col min="16" max="16" width="16.351600646972656" hidden="0" customWidth="1"/>
@@ -994,7 +994,6 @@
       <x:c r="L1" s="99"/>
       <x:c r="M1" s="100"/>
       <x:c r="N1" s="100"/>
-      <x:c r="O1" s="100"/>
     </x:row>
     <x:row r="2" ht="22.350000381469727" customHeight="1">
       <x:c r="A2" s="80" t="str">
@@ -1004,92 +1003,87 @@
         <x:v>本题的标准答案</x:v>
       </x:c>
       <x:c r="C2" s="80" t="str">
-        <x:v>评分备注</x:v>
-      </x:c>
-      <x:c r="D2" s="80" t="str">
         <x:v>gpt-5-6-sol</x:v>
       </x:c>
+      <x:c r="D2" s="80"/>
       <x:c r="E2" s="81"/>
-      <x:c r="F2" s="80"/>
-      <x:c r="G2" s="81" t="str">
+      <x:c r="F2" s="80" t="str">
         <x:v>gpt-5-6-sol</x:v>
       </x:c>
+      <x:c r="G2" s="81"/>
       <x:c r="H2" s="80"/>
-      <x:c r="I2" s="81"/>
-      <x:c r="J2" s="80" t="str">
+      <x:c r="I2" s="81" t="str">
         <x:v>qwen3-8-flash</x:v>
       </x:c>
+      <x:c r="J2" s="80"/>
       <x:c r="K2" s="81"/>
-      <x:c r="L2" s="81"/>
-      <x:c r="M2" s="31" t="str">
+      <x:c r="L2" s="81" t="str">
         <x:v>qwen3-8-flash</x:v>
       </x:c>
+      <x:c r="M2" s="31"/>
       <x:c r="N2" s="31"/>
-      <x:c r="O2" s="31"/>
     </x:row>
     <x:row r="3" ht="20" customHeight="1">
       <x:c r="A3" s="81"/>
       <x:c r="B3" s="81"/>
-      <x:c r="C3" s="81"/>
-      <x:c r="D3" s="80" t="str">
+      <x:c r="C3" s="81" t="str">
         <x:v>skill-on</x:v>
       </x:c>
+      <x:c r="D3" s="80"/>
       <x:c r="E3" s="81"/>
-      <x:c r="F3" s="80"/>
-      <x:c r="G3" s="81" t="str">
+      <x:c r="F3" s="80" t="str">
         <x:v>skill-off</x:v>
       </x:c>
+      <x:c r="G3" s="81"/>
       <x:c r="H3" s="80"/>
-      <x:c r="I3" s="81"/>
-      <x:c r="J3" s="80" t="str">
+      <x:c r="I3" s="81" t="str">
         <x:v>skill-on</x:v>
       </x:c>
+      <x:c r="J3" s="80"/>
       <x:c r="K3" s="81"/>
-      <x:c r="L3" s="81"/>
-      <x:c r="M3" s="31" t="str">
+      <x:c r="L3" s="81" t="str">
         <x:v>skill-off</x:v>
       </x:c>
+      <x:c r="M3" s="31"/>
       <x:c r="N3" s="31"/>
-      <x:c r="O3" s="31"/>
     </x:row>
     <x:row r="4" ht="22.5" customHeight="1">
       <x:c r="A4" s="82"/>
       <x:c r="B4" s="82"/>
-      <x:c r="C4" s="82"/>
+      <x:c r="C4" s="82" t="str">
+        <x:v>作答结果</x:v>
+      </x:c>
       <x:c r="D4" s="95" t="str">
+        <x:v>v0.9.2 得分</x:v>
+      </x:c>
+      <x:c r="E4" s="95" t="str">
+        <x:v>v0.9.3 得分</x:v>
+      </x:c>
+      <x:c r="F4" s="95" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="E4" s="95" t="str">
+      <x:c r="G4" s="95" t="str">
         <x:v>v0.9.2 得分</x:v>
       </x:c>
-      <x:c r="F4" s="95" t="str">
+      <x:c r="H4" s="95" t="str">
         <x:v>v0.9.3 得分</x:v>
       </x:c>
-      <x:c r="G4" s="95" t="str">
+      <x:c r="I4" s="95" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="H4" s="95" t="str">
+      <x:c r="J4" s="95" t="str">
         <x:v>v0.9.2 得分</x:v>
       </x:c>
-      <x:c r="I4" s="95" t="str">
+      <x:c r="K4" s="95" t="str">
         <x:v>v0.9.3 得分</x:v>
       </x:c>
-      <x:c r="J4" s="95" t="str">
+      <x:c r="L4" s="82" t="str">
         <x:v>作答结果</x:v>
       </x:c>
-      <x:c r="K4" s="95" t="str">
+      <x:c r="M4" s="33" t="str">
         <x:v>v0.9.2 得分</x:v>
       </x:c>
-      <x:c r="L4" s="82" t="str">
-        <x:v>v0.9.3 得分</x:v>
-      </x:c>
-      <x:c r="M4" s="33" t="str">
-        <x:v>作答结果</x:v>
-      </x:c>
       <x:c r="N4" s="33" t="str">
-        <x:v>v0.9.2 得分</x:v>
-      </x:c>
-      <x:c r="O4" s="33" t="str">
         <x:v>v0.9.3 得分</x:v>
       </x:c>
     </x:row>
@@ -1101,42 +1095,39 @@
         <x:v>{"answer":0.258031679,"unit":"kJ/mol"}</x:v>
       </x:c>
       <x:c r="C5" s="92" t="str">
-        <x:v>free_energy_difference：标准答案 0.258031679 kJ/mol；linear_goal_v2。满分：x=0.258031679。部分分：|x-0.258031679|&lt;10 按距离线性递减。0分：|x-0.258031679|≥10、单位不匹配或值无效。</x:v>
-      </x:c>
-      <x:c r="D5" s="92" t="str">
         <x:v>{"answer":0.0799,"unit":"kJ/mol"}</x:v>
       </x:c>
+      <x:c r="D5" s="92" t="n">
+        <x:v>0.982187</x:v>
+      </x:c>
       <x:c r="E5" s="23" t="n">
-        <x:v>0.982187</x:v>
-      </x:c>
-      <x:c r="F5" s="23" t="n">
         <x:v>0.977733540125</x:v>
       </x:c>
-      <x:c r="G5" s="92" t="str">
+      <x:c r="F5" s="23" t="str">
         <x:v>{"answer":90.35,"unit":"kJ/mol"}</x:v>
       </x:c>
+      <x:c r="G5" s="92" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="H5" s="23" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I5" s="23" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J5" s="92" t="str">
+      <x:c r="I5" s="23" t="str">
         <x:v>{"answer":0.08,"unit":"kJ/mol"}</x:v>
       </x:c>
+      <x:c r="J5" s="92" t="n">
+        <x:v>0.982197</x:v>
+      </x:c>
       <x:c r="K5" s="23" t="n">
-        <x:v>0.982197</x:v>
-      </x:c>
-      <x:c r="L5" s="23" t="n">
         <x:v>0.977746040125</x:v>
       </x:c>
-      <x:c r="M5" s="101" t="str">
+      <x:c r="L5" s="23" t="str">
         <x:v>{"answer":2.81,"unit":"kJ/mol"}</x:v>
       </x:c>
+      <x:c r="M5" s="101" t="n">
+        <x:v>0.744803</x:v>
+      </x:c>
       <x:c r="N5" s="103" t="n">
-        <x:v>0.744803</x:v>
-      </x:c>
-      <x:c r="O5" s="103" t="n">
         <x:v>0.681003959875</x:v>
       </x:c>
     </x:row>
@@ -1148,42 +1139,39 @@
         <x:v>{"answers":[{"property":"potential_energy_difference","value":0.079,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
       <x:c r="C6" s="93" t="str">
-        <x:v>potential_energy_difference：标准答案 0.079 eV，容差 ±1；ambient_pressure_phase：标准答案 alpha，精确匹配；high_pressure_phase：标准答案 beta，精确匹配。版本 linear_goal_v2。各 comparison group 取组内最低字段分，再对两组算术平均。</x:v>
-      </x:c>
-      <x:c r="D6" s="93" t="str">
         <x:v>{"answers":[{"property":"potential_energy_difference","value":7.299201259709321,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
       </x:c>
+      <x:c r="D6" s="93" t="n">
+        <x:v>0.666667</x:v>
+      </x:c>
       <x:c r="E6" s="24" t="n">
+        <x:v>0.6666666666666666</x:v>
+      </x:c>
+      <x:c r="F6" s="24" t="str">
+        <x:v>{"answers":[{"property":"potential_energy_difference","value":5.50986,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
+      </x:c>
+      <x:c r="G6" s="93" t="n">
         <x:v>0.666667</x:v>
       </x:c>
-      <x:c r="F6" s="24" t="n">
+      <x:c r="H6" s="24" t="n">
         <x:v>0.6666666666666666</x:v>
       </x:c>
-      <x:c r="G6" s="93" t="str">
-        <x:v>{"answers":[{"property":"potential_energy_difference","value":5.50986,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
-      </x:c>
-      <x:c r="H6" s="24" t="n">
+      <x:c r="I6" s="24" t="str">
+        <x:v>{"answers":[{"property":"potential_energy_difference","value":5.51,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
+      </x:c>
+      <x:c r="J6" s="93" t="n">
         <x:v>0.666667</x:v>
       </x:c>
-      <x:c r="I6" s="24" t="n">
+      <x:c r="K6" s="24" t="n">
         <x:v>0.6666666666666666</x:v>
       </x:c>
-      <x:c r="J6" s="93" t="str">
-        <x:v>{"answers":[{"property":"potential_energy_difference","value":5.51,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
-      </x:c>
-      <x:c r="K6" s="24" t="n">
+      <x:c r="L6" s="24" t="str">
+        <x:v>{"answers":[{"property":"potential_energy_difference","value":7.17,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
+      </x:c>
+      <x:c r="M6" s="102" t="n">
         <x:v>0.666667</x:v>
       </x:c>
-      <x:c r="L6" s="24" t="n">
-        <x:v>0.6666666666666666</x:v>
-      </x:c>
-      <x:c r="M6" s="102" t="str">
-        <x:v>{"answers":[{"property":"potential_energy_difference","value":7.17,"unit":"eV"},{"property":"ambient_pressure_phase","value":"alpha"},{"property":"high_pressure_phase","value":"beta"}]}</x:v>
-      </x:c>
       <x:c r="N6" s="104" t="n">
-        <x:v>0.666667</x:v>
-      </x:c>
-      <x:c r="O6" s="104" t="n">
         <x:v>0.6666666666666666</x:v>
       </x:c>
     </x:row>
@@ -1195,42 +1183,39 @@
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
       <x:c r="C7" s="93" t="str">
-        <x:v>hydrogen_bond_count：标准答案 12 count；linear_goal_v2。满分：x=12。部分分：|x-12|&lt;3 按距离线性递减。0分：|x-12|≥3、单位不匹配或值无效。</x:v>
-      </x:c>
-      <x:c r="D7" s="93" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
+      <x:c r="D7" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="E7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F7" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G7" s="93" t="str">
+      <x:c r="F7" s="24" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
+      <x:c r="G7" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="H7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I7" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J7" s="93" t="str">
+      <x:c r="I7" s="24" t="str">
         <x:v>{"answer":12,"unit":"count"}</x:v>
       </x:c>
+      <x:c r="J7" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="K7" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L7" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M7" s="102" t="str">
+      <x:c r="L7" s="24" t="str">
         <x:v>{"answer":10,"unit":"count"}</x:v>
       </x:c>
+      <x:c r="M7" s="102" t="n">
+        <x:v>0.333333</x:v>
+      </x:c>
       <x:c r="N7" s="104" t="n">
-        <x:v>0.333333</x:v>
-      </x:c>
-      <x:c r="O7" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1242,42 +1227,39 @@
         <x:v>{"answers":[{"property":"frequency_1","value":1208.10,"unit":"cm^-1"},{"property":"frequency_2","value":1685.56,"unit":"cm^-1"}]}</x:v>
       </x:c>
       <x:c r="C8" s="93" t="str">
-        <x:v>top_two_frequencies：两项标准答案分别为 1208.10 和 1685.56 cm^-1，各容差 ±100；采用无序最佳一一匹配，comparison group 取匹配后的最低字段分。版本 linear_goal_v2。</x:v>
-      </x:c>
-      <x:c r="D8" s="93" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":435.81,"unit":"cm^-1"},{"property":"frequency_2","value":1585.74,"unit":"cm^-1"},{"property":"frequency_3","value":1592.57,"unit":"cm^-1"}]}</x:v>
       </x:c>
+      <x:c r="D8" s="93" t="n">
+        <x:v>0.0009</x:v>
+      </x:c>
       <x:c r="E8" s="24" t="n">
-        <x:v>0.0009</x:v>
-      </x:c>
-      <x:c r="F8" s="24" t="n">
         <x:v>0.000900000000000345</x:v>
       </x:c>
-      <x:c r="G8" s="93" t="str">
+      <x:c r="F8" s="24" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1585.71,"unit":"cm^-1"},{"property":"frequency_2","value":436.11,"unit":"cm^-1"},{"property":"frequency_3","value":1592.37,"unit":"cm^-1"}]}</x:v>
       </x:c>
+      <x:c r="G8" s="93" t="n">
+        <x:v>0.00075</x:v>
+      </x:c>
       <x:c r="H8" s="24" t="n">
-        <x:v>0.00075</x:v>
-      </x:c>
-      <x:c r="I8" s="24" t="n">
         <x:v>0.0007500000000004725</x:v>
       </x:c>
-      <x:c r="J8" s="93" t="str">
+      <x:c r="I8" s="24" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1584.79,"unit":"cm^-1"},{"property":"frequency_2","value":433.87,"unit":"cm^-1"},{"property":"frequency_3","value":1592.2,"unit":"cm^-1"}]}</x:v>
       </x:c>
+      <x:c r="J8" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="K8" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L8" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M8" s="102" t="str">
+      <x:c r="L8" s="24" t="str">
         <x:v>{"answers":[{"property":"frequency_1","value":1624.6,"unit":"cm^-1"},{"property":"frequency_2","value":1246.4,"unit":"cm^-1"},{"property":"frequency_3","value":843.1,"unit":"cm^-1"}]}</x:v>
       </x:c>
+      <x:c r="M8" s="102" t="n">
+        <x:v>0.5037</x:v>
+      </x:c>
       <x:c r="N8" s="104" t="n">
-        <x:v>0.5037</x:v>
-      </x:c>
-      <x:c r="O8" s="104" t="n">
         <x:v>0.5036999999999989</x:v>
       </x:c>
     </x:row>
@@ -1289,42 +1271,39 @@
         <x:v>{"answer":1.44728,"unit":"g/cm^3"}</x:v>
       </x:c>
       <x:c r="C9" s="93" t="str">
-        <x:v>crystal_density：标准答案 1.44728 g/cm^3；linear_goal_v2。满分：x=1.44728。部分分：|x-1.44728|&lt;0.2 按距离线性递减。0分：|x-1.44728|≥0.2、单位不匹配或值无效。</x:v>
-      </x:c>
-      <x:c r="D9" s="93" t="str">
         <x:v>{"answer":1.55,"unit":"g/cm^3"}</x:v>
       </x:c>
+      <x:c r="D9" s="93" t="n">
+        <x:v>0.4864</x:v>
+      </x:c>
       <x:c r="E9" s="24" t="n">
-        <x:v>0.4864</x:v>
-      </x:c>
-      <x:c r="F9" s="24" t="n">
         <x:v>0.2902548228400852</x:v>
       </x:c>
-      <x:c r="G9" s="93" t="str">
+      <x:c r="F9" s="24" t="str">
         <x:v>{"answer":1.56,"unit":"g/cm^3"}</x:v>
       </x:c>
+      <x:c r="G9" s="93" t="n">
+        <x:v>0.4364</x:v>
+      </x:c>
       <x:c r="H9" s="24" t="n">
-        <x:v>0.4364</x:v>
-      </x:c>
-      <x:c r="I9" s="24" t="n">
         <x:v>0.2211596926648599</x:v>
       </x:c>
-      <x:c r="J9" s="93" t="str">
+      <x:c r="I9" s="24" t="str">
         <x:v>{"answer":1.47,"unit":"g/cm^3"}</x:v>
       </x:c>
+      <x:c r="J9" s="93" t="n">
+        <x:v>0.8864</x:v>
+      </x:c>
       <x:c r="K9" s="24" t="n">
-        <x:v>0.8864</x:v>
-      </x:c>
-      <x:c r="L9" s="24" t="n">
         <x:v>0.8430158642418877</x:v>
       </x:c>
-      <x:c r="M9" s="102" t="str">
+      <x:c r="L9" s="24" t="str">
         <x:v>{"answer":1.28,"unit":"g/cm^3"}</x:v>
       </x:c>
+      <x:c r="M9" s="102" t="n">
+        <x:v>0.1636</x:v>
+      </x:c>
       <x:c r="N9" s="104" t="n">
-        <x:v>0.1636</x:v>
-      </x:c>
-      <x:c r="O9" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1336,42 +1315,39 @@
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
       <x:c r="C10" s="93" t="str">
-        <x:v>cocrystal_ratio：标准答案 1:1；版本 linear_goal_v2。精确匹配得 1 分；1:2 或 2:1 得 0.5 分；其他结果得 0 分。</x:v>
-      </x:c>
-      <x:c r="D10" s="93" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
+      <x:c r="D10" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="E10" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F10" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G10" s="93" t="str">
+      <x:c r="F10" s="24" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
+      <x:c r="G10" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="H10" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I10" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="J10" s="93" t="str">
+      <x:c r="I10" s="24" t="str">
         <x:v>{"answer":"1:1"}</x:v>
       </x:c>
+      <x:c r="J10" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="K10" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L10" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M10" s="102" t="str">
+      <x:c r="L10" s="24" t="str">
         <x:v>{"answer":"1:2"}</x:v>
       </x:c>
+      <x:c r="M10" s="102" t="n">
+        <x:v>0.5</x:v>
+      </x:c>
       <x:c r="N10" s="104" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="O10" s="104" t="n">
         <x:v>0.5</x:v>
       </x:c>
     </x:row>
@@ -1383,42 +1359,39 @@
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormC"},{"property":"crossover_temperature","value":343.15,"unit":"K"}]}</x:v>
       </x:c>
       <x:c r="C11" s="93" t="str">
-        <x:v>lower_free_energy_at_0k：标准答案 FormC，精确匹配；crossover_temperature：标准答案 343.15 K，容差 ±200。版本 linear_goal_v2。题目分取全部字段中的最低值。</x:v>
-      </x:c>
-      <x:c r="D11" s="93" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":3016,"unit":"K"}]}</x:v>
       </x:c>
+      <x:c r="D11" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E11" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F11" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G11" s="93" t="str">
+      <x:c r="F11" s="24" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormC"},{"property":"crossover_temperature","value":943,"unit":"K"}]}</x:v>
+      </x:c>
+      <x:c r="G11" s="93" t="n">
+        <x:v>0.5</x:v>
       </x:c>
       <x:c r="H11" s="24" t="n">
         <x:v>0.5</x:v>
       </x:c>
-      <x:c r="I11" s="24" t="n">
-        <x:v>0.5</x:v>
-      </x:c>
-      <x:c r="J11" s="93" t="str">
+      <x:c r="I11" s="24" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":428.5,"unit":"K"}]}</x:v>
       </x:c>
+      <x:c r="J11" s="93" t="n">
+        <x:v>0.286625</x:v>
+      </x:c>
       <x:c r="K11" s="24" t="n">
-        <x:v>0.286625</x:v>
-      </x:c>
-      <x:c r="L11" s="24" t="n">
         <x:v>0.07324999999999987</x:v>
       </x:c>
-      <x:c r="M11" s="102" t="str">
+      <x:c r="L11" s="24" t="str">
         <x:v>{"answers":[{"property":"lower_free_energy_at_0k","value":"FormA"},{"property":"crossover_temperature","value":300,"unit":"K"}]}</x:v>
       </x:c>
+      <x:c r="M11" s="102" t="n">
+        <x:v>0.392125</x:v>
+      </x:c>
       <x:c r="N11" s="104" t="n">
-        <x:v>0.392125</x:v>
-      </x:c>
-      <x:c r="O11" s="104" t="n">
         <x:v>0.2842500000000001</x:v>
       </x:c>
     </x:row>
@@ -1430,42 +1403,39 @@
         <x:v>{"answers":[{"property":"interaction_energy","value":-69.04,"unit":"kcal/mol"},{"property":"binding_energy","value":-58.15,"unit":"kcal/mol"}]}</x:v>
       </x:c>
       <x:c r="C12" s="93" t="str">
-        <x:v>interaction_energy 与 binding_energy：标准答案分别为 -69.04 和 -58.15 kcal/mol；先取绝对值再按 ±20 线性评分。版本 linear_goal_v2。题目分取两字段最低值。</x:v>
-      </x:c>
-      <x:c r="D12" s="93" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.4733,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.3678,"unit":"kcal/mol"}]}</x:v>
       </x:c>
+      <x:c r="D12" s="93" t="n">
+        <x:v>0.933723</x:v>
+      </x:c>
       <x:c r="E12" s="24" t="n">
-        <x:v>0.933723</x:v>
-      </x:c>
-      <x:c r="F12" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G12" s="93" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="F12" s="24" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.47,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.38,"unit":"kcal/mol"}]}</x:v>
       </x:c>
+      <x:c r="G12" s="93" t="n">
+        <x:v>0.9335</x:v>
+      </x:c>
       <x:c r="H12" s="24" t="n">
-        <x:v>0.9335</x:v>
-      </x:c>
-      <x:c r="I12" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J12" s="93" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I12" s="24" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.45,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.37,"unit":"kcal/mol"}]}</x:v>
       </x:c>
+      <x:c r="J12" s="93" t="n">
+        <x:v>0.93425</x:v>
+      </x:c>
       <x:c r="K12" s="24" t="n">
-        <x:v>0.93425</x:v>
-      </x:c>
-      <x:c r="L12" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M12" s="102" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L12" s="24" t="str">
         <x:v>{"answers":[{"property":"interaction_energy","value":-70.49,"unit":"kcal/mol"},{"property":"binding_energy","value":-59.38,"unit":"kcal/mol"}]}</x:v>
       </x:c>
+      <x:c r="M12" s="102" t="n">
+        <x:v>0.933</x:v>
+      </x:c>
       <x:c r="N12" s="104" t="n">
-        <x:v>0.933</x:v>
-      </x:c>
-      <x:c r="O12" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1477,42 +1447,39 @@
         <x:v>{"answer":7.26,"unit":"eV"}</x:v>
       </x:c>
       <x:c r="C13" s="93" t="str">
-        <x:v>homo_lumo_gap：标准答案 7.26 eV；linear_goal_v2。满分：x=7.26。部分分：|x-7.26|&lt;2 按距离线性递减。0分：|x-7.26|≥2、单位不匹配或值无效。</x:v>
-      </x:c>
-      <x:c r="D13" s="93" t="str">
         <x:v>{"answer":3.558797467914,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="D13" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E13" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F13" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G13" s="93" t="str">
+      <x:c r="F13" s="24" t="str">
         <x:v>{"answer":3.559175368755,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="G13" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="H13" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I13" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J13" s="93" t="str">
+      <x:c r="I13" s="24" t="str">
         <x:v>{"answer":3.5845,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="J13" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="K13" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L13" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M13" s="102" t="str">
+      <x:c r="L13" s="24" t="str">
         <x:v>{"answer":3.584,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="M13" s="102" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="N13" s="104" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O13" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1524,42 +1491,39 @@
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.029,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.485,"unit":"angstrom"}]}</x:v>
       </x:c>
       <x:c r="C14" s="93" t="str">
-        <x:v>oh_bond_distance 与 h_o_contact_distance：标准答案分别为 1.029 和 1.485 angstrom；先取绝对值再按 ±0.3 线性评分。版本 linear_goal_v2。题目分取两字段最低值。</x:v>
-      </x:c>
-      <x:c r="D14" s="93" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
+      <x:c r="D14" s="93" t="n">
+        <x:v>0.776667</x:v>
+      </x:c>
       <x:c r="E14" s="24" t="n">
+        <x:v>0.6650000000000003</x:v>
+      </x:c>
+      <x:c r="F14" s="24" t="str">
+        <x:v>{"answers":[{"property":"oh_bond_distance","value":1.001520301,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.594671850,"unit":"angstrom"}]}</x:v>
+      </x:c>
+      <x:c r="G14" s="93" t="n">
+        <x:v>0.771414</x:v>
+      </x:c>
+      <x:c r="H14" s="24" t="n">
+        <x:v>0.6571211275000007</x:v>
+      </x:c>
+      <x:c r="I14" s="24" t="str">
+        <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
+      </x:c>
+      <x:c r="J14" s="93" t="n">
         <x:v>0.776667</x:v>
       </x:c>
-      <x:c r="F14" s="24" t="n">
+      <x:c r="K14" s="24" t="n">
         <x:v>0.6650000000000003</x:v>
       </x:c>
-      <x:c r="G14" s="93" t="str">
-        <x:v>{"answers":[{"property":"oh_bond_distance","value":1.001520301,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.594671850,"unit":"angstrom"}]}</x:v>
-      </x:c>
-      <x:c r="H14" s="24" t="n">
-        <x:v>0.771414</x:v>
-      </x:c>
-      <x:c r="I14" s="24" t="n">
-        <x:v>0.6571211275000007</x:v>
-      </x:c>
-      <x:c r="J14" s="93" t="str">
+      <x:c r="L14" s="24" t="str">
         <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
       </x:c>
-      <x:c r="K14" s="24" t="n">
+      <x:c r="M14" s="102" t="n">
         <x:v>0.776667</x:v>
       </x:c>
-      <x:c r="L14" s="24" t="n">
-        <x:v>0.6650000000000003</x:v>
-      </x:c>
-      <x:c r="M14" s="102" t="str">
-        <x:v>{"answers":[{"property":"oh_bond_distance","value":1.002,"unit":"angstrom"},{"property":"h_o_contact_distance","value":1.592,"unit":"angstrom"}]}</x:v>
-      </x:c>
       <x:c r="N14" s="104" t="n">
-        <x:v>0.776667</x:v>
-      </x:c>
-      <x:c r="O14" s="104" t="n">
         <x:v>0.6650000000000003</x:v>
       </x:c>
     </x:row>
@@ -1571,42 +1535,39 @@
         <x:v>{"answer":1.713,"unit":"ratio"}</x:v>
       </x:c>
       <x:c r="C15" s="93" t="str">
-        <x:v>accessible_to_inaccessible_volume_ratio：标准答案 1.713 ratio；linear_goal_v2。满分：x=1.713。部分分：|x-1.713|&lt;0.5 按距离线性递减。0分：|x-1.713|≥0.5、单位不匹配或值无效。</x:v>
-      </x:c>
-      <x:c r="D15" s="93" t="str">
         <x:v>{"answer":0.0443,"unit":"ratio"}</x:v>
       </x:c>
+      <x:c r="D15" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E15" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F15" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G15" s="93" t="str">
+      <x:c r="F15" s="24" t="str">
         <x:v>{"answer":0.07236,"unit":"ratio"}</x:v>
       </x:c>
+      <x:c r="G15" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="H15" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I15" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J15" s="93" t="str">
+      <x:c r="I15" s="24" t="str">
         <x:v>{"answer":0.076,"unit":"ratio"}</x:v>
       </x:c>
+      <x:c r="J15" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="K15" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L15" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M15" s="102" t="str">
+      <x:c r="L15" s="24" t="str">
         <x:v>{"answer":0.0724,"unit":"ratio"}</x:v>
       </x:c>
+      <x:c r="M15" s="102" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="N15" s="104" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O15" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1618,42 +1579,39 @@
         <x:v>{"answer":2.521,"unit":"angstrom"}</x:v>
       </x:c>
       <x:c r="C16" s="93" t="str">
-        <x:v>carboxyl_hydrogen_distance：标准答案 2.521 angstrom；linear_goal_v2。满分：x=2.521。部分分：|x-2.521|&lt;0.5 按距离线性递减。0分：|x-2.521|≥0.5、单位不匹配或值无效。</x:v>
-      </x:c>
-      <x:c r="D16" s="93" t="str">
         <x:v>{"answer":2.5212,"unit":"angstrom"}</x:v>
       </x:c>
+      <x:c r="D16" s="93" t="n">
+        <x:v>0.9996</x:v>
+      </x:c>
       <x:c r="E16" s="24" t="n">
-        <x:v>0.9996</x:v>
-      </x:c>
-      <x:c r="F16" s="24" t="n">
         <x:v>0.9990000000000001</x:v>
       </x:c>
-      <x:c r="G16" s="93" t="str">
+      <x:c r="F16" s="24" t="str">
         <x:v>{"answer":2.5183,"unit":"angstrom"}</x:v>
       </x:c>
+      <x:c r="G16" s="93" t="n">
+        <x:v>0.9946</x:v>
+      </x:c>
       <x:c r="H16" s="24" t="n">
-        <x:v>0.9946</x:v>
-      </x:c>
-      <x:c r="I16" s="24" t="n">
         <x:v>0.9865000000000004</x:v>
       </x:c>
-      <x:c r="J16" s="93" t="str">
+      <x:c r="I16" s="24" t="str">
         <x:v>{"answer":2.52,"unit":"angstrom"}</x:v>
       </x:c>
+      <x:c r="J16" s="93" t="n">
+        <x:v>0.998</x:v>
+      </x:c>
       <x:c r="K16" s="24" t="n">
-        <x:v>0.998</x:v>
-      </x:c>
-      <x:c r="L16" s="24" t="n">
         <x:v>0.9950000000000006</x:v>
       </x:c>
-      <x:c r="M16" s="102" t="str">
+      <x:c r="L16" s="24" t="str">
         <x:v>{"answer":2.7043,"unit":"angstrom"}</x:v>
       </x:c>
+      <x:c r="M16" s="102" t="n">
+        <x:v>0.6334</x:v>
+      </x:c>
       <x:c r="N16" s="104" t="n">
-        <x:v>0.6334</x:v>
-      </x:c>
-      <x:c r="O16" s="104" t="n">
         <x:v>0.08349999999999991</x:v>
       </x:c>
     </x:row>
@@ -1665,42 +1623,39 @@
         <x:v>{"answer":-17.11,"unit":"kcal/mol"}</x:v>
       </x:c>
       <x:c r="C17" s="93" t="str">
-        <x:v>halogen_bond_interaction_energy：标准答案 -17.11 kcal/mol；先取绝对值再按 ±5 线性评分。版本 linear_goal_v2。0分：绝对值误差≥5、单位不匹配或值无效。</x:v>
-      </x:c>
-      <x:c r="D17" s="93" t="str">
         <x:v>{"answer":-17.11,"unit":"kcal/mol"}</x:v>
       </x:c>
+      <x:c r="D17" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="E17" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F17" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G17" s="93" t="str">
+      <x:c r="F17" s="24" t="str">
         <x:v>{"answer":-19.17,"unit":"kcal/mol"}</x:v>
       </x:c>
+      <x:c r="G17" s="93" t="n">
+        <x:v>0.588</x:v>
+      </x:c>
       <x:c r="H17" s="24" t="n">
-        <x:v>0.588</x:v>
-      </x:c>
-      <x:c r="I17" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J17" s="93" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I17" s="24" t="str">
         <x:v>{"answer":-15.5969,"unit":"kcal/mol"}</x:v>
       </x:c>
+      <x:c r="J17" s="93" t="n">
+        <x:v>0.69738</x:v>
+      </x:c>
       <x:c r="K17" s="24" t="n">
-        <x:v>0.69738</x:v>
-      </x:c>
-      <x:c r="L17" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M17" s="102" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L17" s="24" t="str">
         <x:v>{"answer":-16.5,"unit":"kcal/mol"}</x:v>
       </x:c>
+      <x:c r="M17" s="102" t="n">
+        <x:v>0.878</x:v>
+      </x:c>
       <x:c r="N17" s="104" t="n">
-        <x:v>0.878</x:v>
-      </x:c>
-      <x:c r="O17" s="104" t="n">
         <x:v>0.39000000000000057</x:v>
       </x:c>
     </x:row>
@@ -1712,42 +1667,39 @@
         <x:v>{"answer":5.7,"unit":"pKa"}</x:v>
       </x:c>
       <x:c r="C18" s="93" t="str">
-        <x:v>pka：标准答案 5.7 pKa；linear_goal_v2。满分：x=5.7。部分分：|x-5.7|&lt;2 按距离线性递减。0分：|x-5.7|≥2、单位不匹配或值无效。</x:v>
-      </x:c>
-      <x:c r="D18" s="93" t="str">
         <x:v>{"answer":5.0,"unit":"pKa"}</x:v>
       </x:c>
+      <x:c r="D18" s="93" t="n">
+        <x:v>0.65</x:v>
+      </x:c>
       <x:c r="E18" s="24" t="n">
-        <x:v>0.65</x:v>
-      </x:c>
-      <x:c r="F18" s="24" t="n">
         <x:v>0.6499999999999999</x:v>
       </x:c>
-      <x:c r="G18" s="93" t="str">
+      <x:c r="F18" s="24" t="str">
         <x:v>{"answer":6.33,"unit":"pKa"}</x:v>
+      </x:c>
+      <x:c r="G18" s="93" t="n">
+        <x:v>0.685</x:v>
       </x:c>
       <x:c r="H18" s="24" t="n">
         <x:v>0.685</x:v>
       </x:c>
-      <x:c r="I18" s="24" t="n">
-        <x:v>0.685</x:v>
-      </x:c>
-      <x:c r="J18" s="93" t="str">
+      <x:c r="I18" s="24" t="str">
         <x:v>{"answer":5.7,"unit":"pKa"}</x:v>
       </x:c>
+      <x:c r="J18" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="K18" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L18" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M18" s="102" t="str">
+      <x:c r="L18" s="24" t="str">
         <x:v>{"answer":6.8,"unit":"pKa"}</x:v>
       </x:c>
+      <x:c r="M18" s="102" t="n">
+        <x:v>0.45</x:v>
+      </x:c>
       <x:c r="N18" s="104" t="n">
-        <x:v>0.45</x:v>
-      </x:c>
-      <x:c r="O18" s="104" t="n">
         <x:v>0.4500000000000002</x:v>
       </x:c>
     </x:row>
@@ -1759,42 +1711,39 @@
         <x:v>{"answer":0.00734,"unit":"eV"}</x:v>
       </x:c>
       <x:c r="C19" s="93" t="str">
-        <x:v>spin_orbit_coupling_matrix_element：标准答案 0.00734 eV；对 x 与标准答案分别取 log10，在 log10 空间按 ±1 线性评分。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
-      </x:c>
-      <x:c r="D19" s="93" t="str">
         <x:v>{"answer":0.00485,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="D19" s="93" t="n">
+        <x:v>0.820046</x:v>
+      </x:c>
       <x:c r="E19" s="24" t="n">
-        <x:v>0.820046</x:v>
-      </x:c>
-      <x:c r="F19" s="24" t="n">
         <x:v>0.8200456786861929</x:v>
       </x:c>
-      <x:c r="G19" s="93" t="str">
+      <x:c r="F19" s="24" t="str">
         <x:v>{"answer":0.0035,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="G19" s="93" t="n">
+        <x:v>0.678372</x:v>
+      </x:c>
       <x:c r="H19" s="24" t="n">
-        <x:v>0.678372</x:v>
-      </x:c>
-      <x:c r="I19" s="24" t="n">
         <x:v>0.6783719844342051</x:v>
       </x:c>
-      <x:c r="J19" s="93" t="str">
+      <x:c r="I19" s="24" t="str">
         <x:v>{"answer":0.0,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="J19" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="K19" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="L19" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M19" s="102" t="str">
+      <x:c r="L19" s="24" t="str">
         <x:v>{"answer":0.01,"unit":"eV"}</x:v>
       </x:c>
+      <x:c r="M19" s="102" t="n">
+        <x:v>0.865696</x:v>
+      </x:c>
       <x:c r="N19" s="104" t="n">
-        <x:v>0.865696</x:v>
-      </x:c>
-      <x:c r="O19" s="104" t="n">
         <x:v>0.8656960599160706</x:v>
       </x:c>
     </x:row>
@@ -1806,42 +1755,39 @@
         <x:v>{"answer":117000000,"unit":"s^-1"}</x:v>
       </x:c>
       <x:c r="C20" s="93" t="str">
-        <x:v>intersystem_crossing_rate：标准答案 117000000 s^-1；对 x 与标准答案分别取 log10，在 log10 空间按 ±3 线性评分。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
-      </x:c>
-      <x:c r="D20" s="93" t="str">
         <x:v>{"answer":1.2e8,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="D20" s="93" t="n">
+        <x:v>0.996335</x:v>
+      </x:c>
       <x:c r="E20" s="24" t="n">
-        <x:v>0.996335</x:v>
-      </x:c>
-      <x:c r="F20" s="24" t="n">
         <x:v>0.9945023078492685</x:v>
       </x:c>
-      <x:c r="G20" s="93" t="str">
+      <x:c r="F20" s="24" t="str">
         <x:v>{"answer":1.45e8,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="G20" s="93" t="n">
+        <x:v>0.968939</x:v>
+      </x:c>
       <x:c r="H20" s="24" t="n">
-        <x:v>0.968939</x:v>
-      </x:c>
-      <x:c r="I20" s="24" t="n">
         <x:v>0.9534089297555939</x:v>
       </x:c>
-      <x:c r="J20" s="93" t="str">
+      <x:c r="I20" s="24" t="str">
         <x:v>{"answer":1e6,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="J20" s="93" t="n">
+        <x:v>0.310605</x:v>
+      </x:c>
       <x:c r="K20" s="24" t="n">
-        <x:v>0.310605</x:v>
-      </x:c>
-      <x:c r="L20" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="M20" s="102" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="L20" s="24" t="str">
         <x:v>{"answer":100000,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="M20" s="102" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="N20" s="104" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O20" s="104" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -1853,42 +1799,39 @@
         <x:v>{"answer":98,"unit":"s^-1"}</x:v>
       </x:c>
       <x:c r="C21" s="93" t="str">
-        <x:v>phosphorescence_rate：标准答案 98 s^-1；对 x 与标准答案分别取 log10，在 log10 空间下侧容差 2、上侧容差 3，按线性距离递减。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
-      </x:c>
-      <x:c r="D21" s="93" t="str">
         <x:v>{"answer":91.92785,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="D21" s="93" t="n">
+        <x:v>0.986111</x:v>
+      </x:c>
       <x:c r="E21" s="24" t="n">
-        <x:v>0.986111</x:v>
-      </x:c>
-      <x:c r="F21" s="24" t="n">
         <x:v>0.9861105136520333</x:v>
       </x:c>
-      <x:c r="G21" s="93" t="str">
+      <x:c r="F21" s="24" t="str">
         <x:v>{"answer":100.0,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="G21" s="93" t="n">
+        <x:v>0.997075</x:v>
+      </x:c>
       <x:c r="H21" s="24" t="n">
+        <x:v>0.9956130378462474</x:v>
+      </x:c>
+      <x:c r="I21" s="24" t="str">
+        <x:v>{"answer":100,"unit":"s^-1"}</x:v>
+      </x:c>
+      <x:c r="J21" s="93" t="n">
         <x:v>0.997075</x:v>
       </x:c>
-      <x:c r="I21" s="24" t="n">
+      <x:c r="K21" s="24" t="n">
         <x:v>0.9956130378462474</x:v>
       </x:c>
-      <x:c r="J21" s="93" t="str">
-        <x:v>{"answer":100,"unit":"s^-1"}</x:v>
-      </x:c>
-      <x:c r="K21" s="24" t="n">
-        <x:v>0.997075</x:v>
-      </x:c>
-      <x:c r="L21" s="24" t="n">
-        <x:v>0.9956130378462474</x:v>
-      </x:c>
-      <x:c r="M21" s="102" t="str">
+      <x:c r="L21" s="24" t="str">
         <x:v>{"answer":16.9,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="M21" s="102" t="n">
+        <x:v>0.61833</x:v>
+      </x:c>
       <x:c r="N21" s="104" t="n">
-        <x:v>0.61833</x:v>
-      </x:c>
-      <x:c r="O21" s="104" t="n">
         <x:v>0.6183303144605893</x:v>
       </x:c>
     </x:row>
@@ -1900,42 +1843,39 @@
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
       <x:c r="C22" s="93" t="str">
-        <x:v>herzberg_teller_contribution：标准答案 100 percent；linear_goal_v2。下侧容差 10、上侧容差 1，按距离线性递减；0分：低于 90 或高于 101、单位不匹配或值无效。</x:v>
-      </x:c>
-      <x:c r="D22" s="93" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
+      <x:c r="D22" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="E22" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="F22" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="G22" s="93" t="str">
+      <x:c r="F22" s="24" t="str">
         <x:v>{"answer":70,"unit":"percent"}</x:v>
       </x:c>
+      <x:c r="G22" s="93" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="H22" s="24" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I22" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J22" s="93" t="str">
+      <x:c r="I22" s="24" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
+      <x:c r="J22" s="93" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="K22" s="24" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="L22" s="24" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="M22" s="102" t="str">
+      <x:c r="L22" s="24" t="str">
         <x:v>{"answer":100,"unit":"percent"}</x:v>
       </x:c>
+      <x:c r="M22" s="102" t="n">
+        <x:v>1</x:v>
+      </x:c>
       <x:c r="N22" s="104" t="n">
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="O22" s="104" t="n">
         <x:v>1</x:v>
       </x:c>
     </x:row>
@@ -1947,42 +1887,39 @@
         <x:v>{"answer":28400000000,"unit":"s^-1"}</x:v>
       </x:c>
       <x:c r="C23" s="93" t="str">
-        <x:v>intersystem_crossing_rate：标准答案 28400000000 s^-1；对 x 与标准答案分别取 log10，在 log10 空间按 ±3 线性评分。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
-      </x:c>
-      <x:c r="D23" s="93" t="str">
         <x:v>{"answer":2.38e10,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="D23" s="93" t="n">
+        <x:v>0.97442</x:v>
+      </x:c>
       <x:c r="E23" s="24" t="n">
-        <x:v>0.97442</x:v>
-      </x:c>
-      <x:c r="F23" s="24" t="n">
         <x:v>0.9616293085047376</x:v>
       </x:c>
-      <x:c r="G23" s="93" t="str">
+      <x:c r="F23" s="24" t="str">
         <x:v>{"answer":1.6e8,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="G23" s="93" t="n">
+        <x:v>0.250267</x:v>
+      </x:c>
       <x:c r="H23" s="24" t="n">
-        <x:v>0.250267</x:v>
-      </x:c>
-      <x:c r="I23" s="24" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J23" s="93" t="str">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I23" s="24" t="str">
         <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="J23" s="93" t="n">
+        <x:v>0.848894</x:v>
+      </x:c>
       <x:c r="K23" s="24" t="n">
+        <x:v>0.7733408299764815</x:v>
+      </x:c>
+      <x:c r="L23" s="24" t="str">
+        <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
+      </x:c>
+      <x:c r="M23" s="102" t="n">
         <x:v>0.848894</x:v>
       </x:c>
-      <x:c r="L23" s="24" t="n">
-        <x:v>0.7733408299764815</x:v>
-      </x:c>
-      <x:c r="M23" s="102" t="str">
-        <x:v>{"answer":1e10,"unit":"s^-1"}</x:v>
-      </x:c>
       <x:c r="N23" s="104" t="n">
-        <x:v>0.848894</x:v>
-      </x:c>
-      <x:c r="O23" s="104" t="n">
         <x:v>0.7733408299764815</x:v>
       </x:c>
     </x:row>
@@ -1994,40 +1931,37 @@
         <x:v>{"answer":382000000,"unit":"s^-1"}</x:v>
       </x:c>
       <x:c r="C24" s="94" t="str">
-        <x:v>internal_conversion_rate：标准答案 382000000 s^-1；对 x 与标准答案分别取 log10，在 log10 空间按 ±3 线性评分。版本 linear_goal_v2；x≤0、单位不匹配或无效值为0分。</x:v>
-      </x:c>
-      <x:c r="D24" s="94" t="str">
         <x:v>{"answer":1e12,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="D24" s="94" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="E24" s="25" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="F24" s="25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G24" s="94" t="str">
+      <x:c r="F24" s="25" t="str">
         <x:v>{"answer":9.4e11,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="G24" s="94" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="H24" s="25" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="I24" s="25" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="J24" s="98" t="str">
+      <x:c r="I24" s="25" t="str">
         <x:v>{"answer":1.0e9,"unit":"s^-1"}</x:v>
       </x:c>
+      <x:c r="J24" s="98" t="n">
+        <x:v>0.860688</x:v>
+      </x:c>
       <x:c r="K24" s="25" t="n">
-        <x:v>0.860688</x:v>
-      </x:c>
-      <x:c r="L24" s="25" t="n">
         <x:v>0.7910316814558547</x:v>
       </x:c>
-      <x:c r="M24" s="57"/>
+      <x:c r="L24" s="25"/>
+      <x:c r="M24" s="57" t="n">
+        <x:v>0</x:v>
+      </x:c>
       <x:c r="N24" s="43" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="O24" s="43" t="n">
         <x:v>0</x:v>
       </x:c>
     </x:row>
@@ -2036,41 +1970,40 @@
         <x:v>各实验组平均分（未评分项记0分）</x:v>
       </x:c>
       <x:c r="B25" s="91"/>
-      <x:c r="C25" s="91"/>
-      <x:c r="D25" s="96" t="str">
+      <x:c r="C25" s="91" t="str">
         <x:v>平均分</x:v>
       </x:c>
+      <x:c r="D25" s="96" t="n">
+        <x:v>0.663653</x:v>
+      </x:c>
       <x:c r="E25" s="26" t="n">
-        <x:v>0.663653</x:v>
-      </x:c>
-      <x:c r="F25" s="26" t="n">
         <x:v>0.6005921419161993</x:v>
       </x:c>
-      <x:c r="G25" s="97" t="str">
+      <x:c r="F25" s="26" t="str">
         <x:v>平均分</x:v>
       </x:c>
+      <x:c r="G25" s="97" t="n">
+        <x:v>0.523549</x:v>
+      </x:c>
       <x:c r="H25" s="26" t="n">
-        <x:v>0.523549</x:v>
-      </x:c>
-      <x:c r="I25" s="26" t="n">
         <x:v>0.41722957194337873</x:v>
       </x:c>
-      <x:c r="J25" s="96" t="str">
+      <x:c r="I25" s="26" t="str">
         <x:v>平均分</x:v>
       </x:c>
+      <x:c r="J25" s="96" t="n">
+        <x:v>0.662272</x:v>
+      </x:c>
       <x:c r="K25" s="26" t="n">
-        <x:v>0.662272</x:v>
-      </x:c>
-      <x:c r="L25" s="26" t="n">
         <x:v>0.5390332060156069</x:v>
       </x:c>
-      <x:c r="M25" s="61" t="str">
+      <x:c r="L25" s="26" t="str">
         <x:v>平均分</x:v>
       </x:c>
+      <x:c r="M25" s="61" t="n">
+        <x:v>0.515411</x:v>
+      </x:c>
       <x:c r="N25" s="47" t="n">
-        <x:v>0.515411</x:v>
-      </x:c>
-      <x:c r="O25" s="47" t="n">
         <x:v>0.37407439154474037</x:v>
       </x:c>
     </x:row>

</xml_diff>